<commit_message>
Control board Client and eSpark board completed. #70
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Control-Board/eSpark_BOM-Control-Board.xlsx
+++ b/Deliverables/BOM/Control-Board/eSpark_BOM-Control-Board.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25225"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB529AF9-ED5E-4632-946F-077CCFFDF5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="289">
   <si>
     <t>Component list</t>
   </si>
@@ -68,27 +67,15 @@
     <t>C1, C2, C7</t>
   </si>
   <si>
-    <t>C3, C4, C6, C10, C11, C12, C13, C14, C15, C18, C19, C20, C21, C22, C24, C31, C34, C35, C36, C37, C41, C42, C47, C49</t>
-  </si>
-  <si>
     <t>C5</t>
   </si>
   <si>
     <t>C8, C25, C26, C27, C28, C39, C40, C50</t>
   </si>
   <si>
-    <t>C9, C23, C33</t>
-  </si>
-  <si>
-    <t>C16, C30, C32, C43, C45, C46, C48, C51</t>
-  </si>
-  <si>
     <t>C17</t>
   </si>
   <si>
-    <t>C29, C44</t>
-  </si>
-  <si>
     <t>C38</t>
   </si>
   <si>
@@ -116,9 +103,6 @@
     <t>L1</t>
   </si>
   <si>
-    <t>L2</t>
-  </si>
-  <si>
     <t>L3</t>
   </si>
   <si>
@@ -149,12 +133,6 @@
     <t>R4, R5, R6, R12, R18, R19, R22, R23, R25, R27</t>
   </si>
   <si>
-    <t>R7</t>
-  </si>
-  <si>
-    <t>R8, R13, R14, R15, R16, R17, R26</t>
-  </si>
-  <si>
     <t>R10, R11</t>
   </si>
   <si>
@@ -167,9 +145,6 @@
     <t>SB1, SB2, SB3</t>
   </si>
   <si>
-    <t>SW1</t>
-  </si>
-  <si>
     <t>U1</t>
   </si>
   <si>
@@ -248,9 +223,6 @@
     <t>FIXED IND 2.2UH 1.5A 160MOHM SMD</t>
   </si>
   <si>
-    <t>FIXED IND 10UH 360MA 1.32OHM SMD</t>
-  </si>
-  <si>
     <t>500mA 10uH ±20% 320mΩ 0805 Inductors (SMD) ROHS</t>
   </si>
   <si>
@@ -275,9 +247,6 @@
     <t>RES SMD 10K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t>62.5mW Thick Film Resistors 50V ±5% ±200ppm/℃ 1Ω -55℃~+155℃ 0402 Chip Resistor - Surface Mount ROHS</t>
-  </si>
-  <si>
     <t>RES SMD 100K OHM 1% 1/5W 0402</t>
   </si>
   <si>
@@ -365,9 +334,6 @@
     <t>MAKK2016T2R2M</t>
   </si>
   <si>
-    <t>NLCV25T-100K-EFRD</t>
-  </si>
-  <si>
     <t>Ind0805</t>
   </si>
   <si>
@@ -473,9 +439,6 @@
     <t>RC0402FR-0710KL</t>
   </si>
   <si>
-    <t>FRC0402J1R0 TS</t>
-  </si>
-  <si>
     <t>ERJ-PA2F1003X</t>
   </si>
   <si>
@@ -539,9 +502,6 @@
     <t>XFCN</t>
   </si>
   <si>
-    <t>TDK</t>
-  </si>
-  <si>
     <t>microgate</t>
   </si>
   <si>
@@ -554,9 +514,6 @@
     <t>SunLED</t>
   </si>
   <si>
-    <t>FOJAN</t>
-  </si>
-  <si>
     <t>Panasonic</t>
   </si>
   <si>
@@ -650,9 +607,6 @@
     <t>10K</t>
   </si>
   <si>
-    <t>1R</t>
-  </si>
-  <si>
     <t>100K</t>
   </si>
   <si>
@@ -755,9 +709,6 @@
     <t>C424659</t>
   </si>
   <si>
-    <t>C295388</t>
-  </si>
-  <si>
     <t>C281113</t>
   </si>
   <si>
@@ -788,9 +739,6 @@
     <t>C60490</t>
   </si>
   <si>
-    <t>C2906901</t>
-  </si>
-  <si>
     <t>C226678</t>
   </si>
   <si>
@@ -915,12 +863,45 @@
   </si>
   <si>
     <t xml:space="preserve">Need Fresh Quote From Custom Supplier </t>
+  </si>
+  <si>
+    <t>C3, C4, C6, C10, C11, C12, C13, C14, C15, C18, C19, C20, C21, C22, C23, C24, C31, C34, C35, C36, C41, C42, C47, C49</t>
+  </si>
+  <si>
+    <t>C9, C33</t>
+  </si>
+  <si>
+    <t>C16, C32, C43, C45, C46, C48, C51</t>
+  </si>
+  <si>
+    <t>C37</t>
+  </si>
+  <si>
+    <t>CAP CER 100pF 50V C0G 0402</t>
+  </si>
+  <si>
+    <t>Cap 0403</t>
+  </si>
+  <si>
+    <t>GCM1555C1H101JA16D</t>
+  </si>
+  <si>
+    <t>100pF</t>
+  </si>
+  <si>
+    <t>C44</t>
+  </si>
+  <si>
+    <t>R7, R8, R13, R14, R15, R16, R17, R26</t>
+  </si>
+  <si>
+    <t>SW1, SW2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -1135,7 +1116,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="31">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -1497,12 +1478,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="119">
+  <cellXfs count="122">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1766,6 +1762,48 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1792,46 +1830,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="30" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2169,9 +2174,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -2203,8 +2208,8 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="103"/>
-      <c r="K1" s="104"/>
+      <c r="J1" s="117"/>
+      <c r="K1" s="118"/>
     </row>
     <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2220,15 +2225,15 @@
       <c r="G2" s="11"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
-      <c r="J2" s="99"/>
-      <c r="K2" s="99"/>
-      <c r="L2" s="99"/>
-      <c r="M2" s="99"/>
-      <c r="N2" s="99"/>
-      <c r="O2" s="99"/>
-      <c r="P2" s="99"/>
-      <c r="Q2" s="99"/>
-      <c r="R2" s="100"/>
+      <c r="J2" s="113"/>
+      <c r="K2" s="113"/>
+      <c r="L2" s="113"/>
+      <c r="M2" s="113"/>
+      <c r="N2" s="113"/>
+      <c r="O2" s="113"/>
+      <c r="P2" s="113"/>
+      <c r="Q2" s="113"/>
+      <c r="R2" s="114"/>
     </row>
     <row r="3" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
@@ -2252,7 +2257,7 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="97"/>
+      <c r="R3" s="111"/>
     </row>
     <row r="4" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2276,7 +2281,7 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
-      <c r="R4" s="98"/>
+      <c r="R4" s="112"/>
     </row>
     <row r="5" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2300,7 +2305,7 @@
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
       <c r="Q5" s="5"/>
-      <c r="R5" s="98"/>
+      <c r="R5" s="112"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2320,7 +2325,7 @@
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
       <c r="Q6" s="5"/>
-      <c r="R6" s="98"/>
+      <c r="R6" s="112"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2340,7 +2345,7 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="98"/>
+      <c r="R7" s="112"/>
     </row>
     <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2360,7 +2365,7 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="98"/>
+      <c r="R8" s="112"/>
     </row>
     <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2371,49 +2376,49 @@
         <v>10</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E9" s="32" t="s">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="F9" s="33" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="G9" s="32" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="H9" s="77" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="I9" s="33" t="s">
-        <v>218</v>
+        <v>203</v>
       </c>
       <c r="J9" s="32" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="K9" s="77" t="s">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="L9" s="32" t="s">
-        <v>293</v>
+        <v>276</v>
       </c>
       <c r="M9" s="32" t="s">
-        <v>221</v>
+        <v>206</v>
       </c>
       <c r="N9" s="32" t="s">
-        <v>222</v>
+        <v>207</v>
       </c>
       <c r="O9" s="32" t="s">
-        <v>223</v>
+        <v>208</v>
       </c>
       <c r="P9" s="32" t="s">
-        <v>279</v>
+        <v>262</v>
       </c>
       <c r="Q9" s="32" t="s">
-        <v>273</v>
+        <v>256</v>
       </c>
       <c r="R9" s="32" t="s">
-        <v>274</v>
+        <v>257</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
@@ -2426,25 +2431,25 @@
         <v>11</v>
       </c>
       <c r="D10" s="60" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="E10" s="51" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="F10" s="60" t="s">
-        <v>133</v>
-      </c>
-      <c r="G10" s="114" t="s">
-        <v>215</v>
-      </c>
-      <c r="H10" s="106" t="s">
-        <v>161</v>
+        <v>122</v>
+      </c>
+      <c r="G10" s="106" t="s">
+        <v>200</v>
+      </c>
+      <c r="H10" s="98" t="s">
+        <v>149</v>
       </c>
       <c r="I10" s="60" t="s">
-        <v>219</v>
-      </c>
-      <c r="J10" s="51" t="s">
-        <v>189</v>
+        <v>204</v>
+      </c>
+      <c r="J10" s="121" t="s">
+        <v>175</v>
       </c>
       <c r="K10" s="54">
         <v>3</v>
@@ -2457,7 +2462,7 @@
         <v>20</v>
       </c>
       <c r="N10" s="69" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O10" s="42">
         <v>7.2800000000000004E-2</v>
@@ -2472,51 +2477,51 @@
     <row r="11" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="78">
-        <f t="shared" ref="B11:B55" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B54" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="52" t="s">
-        <v>12</v>
+        <v>278</v>
       </c>
       <c r="D11" s="61" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="E11" s="52" t="s">
-        <v>101</v>
-      </c>
-      <c r="F11" s="116" t="s">
-        <v>134</v>
+        <v>91</v>
+      </c>
+      <c r="F11" s="108" t="s">
+        <v>123</v>
       </c>
       <c r="G11" s="52" t="s">
-        <v>225</v>
-      </c>
-      <c r="H11" s="107" t="s">
-        <v>161</v>
+        <v>210</v>
+      </c>
+      <c r="H11" s="99" t="s">
+        <v>149</v>
       </c>
       <c r="I11" s="61" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="J11" s="52" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="K11" s="55">
         <v>24</v>
       </c>
       <c r="L11" s="31">
-        <f t="shared" ref="L11:L55" si="1">K11*5</f>
+        <f t="shared" ref="L11:L54" si="1">K11*5</f>
         <v>120</v>
       </c>
       <c r="M11" s="31">
         <v>150</v>
       </c>
       <c r="N11" s="70" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O11" s="35">
         <v>7.3000000000000001E-3</v>
       </c>
       <c r="P11" s="35">
-        <f t="shared" ref="P11:P55" si="2">O11*M11</f>
+        <f t="shared" ref="P11:P54" si="2">O11*M11</f>
         <v>1.095</v>
       </c>
       <c r="Q11" s="35"/>
@@ -2529,28 +2534,28 @@
         <v>3</v>
       </c>
       <c r="C12" s="53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D12" s="62" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E12" s="53" t="s">
-        <v>102</v>
+        <v>92</v>
       </c>
       <c r="F12" s="62" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="G12" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H12" s="108" t="s">
-        <v>162</v>
+        <v>200</v>
+      </c>
+      <c r="H12" s="100" t="s">
+        <v>150</v>
       </c>
       <c r="I12" s="62" t="s">
-        <v>227</v>
+        <v>212</v>
       </c>
       <c r="J12" s="53" t="s">
-        <v>191</v>
+        <v>177</v>
       </c>
       <c r="K12" s="56">
         <v>1</v>
@@ -2563,7 +2568,7 @@
         <v>20</v>
       </c>
       <c r="N12" s="71" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O12" s="34">
         <v>1.3599999999999999E-2</v>
@@ -2582,28 +2587,28 @@
         <v>4</v>
       </c>
       <c r="C13" s="52" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D13" s="61" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="E13" s="52" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="F13" s="61" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="G13" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H13" s="107" t="s">
-        <v>163</v>
+        <v>200</v>
+      </c>
+      <c r="H13" s="99" t="s">
+        <v>151</v>
       </c>
       <c r="I13" s="61" t="s">
-        <v>229</v>
+        <v>214</v>
       </c>
       <c r="J13" s="52" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="K13" s="55">
         <v>8</v>
@@ -2616,7 +2621,7 @@
         <v>100</v>
       </c>
       <c r="N13" s="70" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O13" s="35">
         <v>1.4E-3</v>
@@ -2635,41 +2640,41 @@
         <v>5</v>
       </c>
       <c r="C14" s="53" t="s">
-        <v>15</v>
+        <v>279</v>
       </c>
       <c r="D14" s="62" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="E14" s="53" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="F14" s="62" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="G14" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H14" s="108" t="s">
-        <v>164</v>
+        <v>200</v>
+      </c>
+      <c r="H14" s="100" t="s">
+        <v>152</v>
       </c>
       <c r="I14" s="62" t="s">
-        <v>228</v>
+        <v>213</v>
       </c>
       <c r="J14" s="53" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="K14" s="56">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" s="30">
         <f t="shared" si="1"/>
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M14" s="30">
         <v>50</v>
       </c>
       <c r="N14" s="72" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O14" s="34">
         <v>1.8499999999999999E-2</v>
@@ -2688,41 +2693,41 @@
         <v>6</v>
       </c>
       <c r="C15" s="52" t="s">
-        <v>16</v>
+        <v>280</v>
       </c>
       <c r="D15" s="61" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="E15" s="52" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="F15" s="61" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="G15" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="H15" s="99" t="s">
+        <v>151</v>
+      </c>
+      <c r="I15" s="61" t="s">
         <v>215</v>
       </c>
-      <c r="H15" s="107" t="s">
-        <v>163</v>
-      </c>
-      <c r="I15" s="61" t="s">
-        <v>230</v>
-      </c>
       <c r="J15" s="52" t="s">
-        <v>194</v>
+        <v>180</v>
       </c>
       <c r="K15" s="55">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L15" s="31">
         <f t="shared" si="1"/>
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="M15" s="31">
         <v>50</v>
       </c>
       <c r="N15" s="70" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O15" s="35">
         <v>6.4000000000000003E-3</v>
@@ -2741,28 +2746,28 @@
         <v>7</v>
       </c>
       <c r="C16" s="53" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D16" s="62" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="E16" s="53" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="F16" s="62" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="G16" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H16" s="108" t="s">
-        <v>161</v>
+        <v>200</v>
+      </c>
+      <c r="H16" s="100" t="s">
+        <v>149</v>
       </c>
       <c r="I16" s="62" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
       <c r="J16" s="53" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="K16" s="56">
         <v>1</v>
@@ -2775,7 +2780,7 @@
         <v>10</v>
       </c>
       <c r="N16" s="72" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O16" s="37">
         <v>4.8899999999999999E-2</v>
@@ -2789,56 +2794,52 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="78">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="C17" s="52" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" s="61" t="s">
-        <v>233</v>
-      </c>
-      <c r="E17" s="52" t="s">
-        <v>101</v>
-      </c>
-      <c r="F17" s="61" t="s">
-        <v>234</v>
-      </c>
-      <c r="G17" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H17" s="107" t="s">
-        <v>163</v>
-      </c>
-      <c r="I17" s="61" t="s">
-        <v>232</v>
-      </c>
-      <c r="J17" s="52" t="s">
-        <v>196</v>
-      </c>
-      <c r="K17" s="55">
-        <v>2</v>
-      </c>
-      <c r="L17" s="31">
+      <c r="B17" s="78"/>
+      <c r="C17" s="53" t="s">
+        <v>281</v>
+      </c>
+      <c r="D17" s="62" t="s">
+        <v>282</v>
+      </c>
+      <c r="E17" s="53" t="s">
+        <v>283</v>
+      </c>
+      <c r="F17" s="62" t="s">
+        <v>284</v>
+      </c>
+      <c r="G17" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="H17" s="62" t="s">
+        <v>285</v>
+      </c>
+      <c r="I17" s="119">
+        <v>1</v>
+      </c>
+      <c r="J17" s="53" t="s">
+        <v>285</v>
+      </c>
+      <c r="K17" s="56">
+        <v>1</v>
+      </c>
+      <c r="L17" s="30">
         <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="M17" s="31">
-        <v>100</v>
-      </c>
-      <c r="N17" s="70" t="s">
-        <v>224</v>
-      </c>
-      <c r="O17" s="35">
-        <v>1.6000000000000001E-3</v>
-      </c>
-      <c r="P17" s="35">
-        <f t="shared" si="2"/>
-        <v>0.16</v>
-      </c>
-      <c r="Q17" s="35"/>
-      <c r="R17" s="35"/>
+        <v>5</v>
+      </c>
+      <c r="M17" s="36">
+        <v>50</v>
+      </c>
+      <c r="N17" s="120" t="s">
+        <v>209</v>
+      </c>
+      <c r="O17" s="37">
+        <v>9.4999999999999998E-3</v>
+      </c>
+      <c r="P17" s="34">
+        <v>0.48</v>
+      </c>
+      <c r="Q17" s="34"/>
+      <c r="R17" s="34"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
@@ -2846,52 +2847,52 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="53" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" s="62" t="s">
-        <v>65</v>
-      </c>
-      <c r="E18" s="53" t="s">
-        <v>101</v>
-      </c>
-      <c r="F18" s="62" t="s">
-        <v>140</v>
-      </c>
-      <c r="G18" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H18" s="108" t="s">
-        <v>161</v>
-      </c>
-      <c r="I18" s="62" t="s">
-        <v>235</v>
-      </c>
-      <c r="J18" s="53" t="s">
-        <v>197</v>
-      </c>
-      <c r="K18" s="56">
+      <c r="C18" s="52" t="s">
+        <v>286</v>
+      </c>
+      <c r="D18" s="61" t="s">
+        <v>218</v>
+      </c>
+      <c r="E18" s="52" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" s="61" t="s">
+        <v>219</v>
+      </c>
+      <c r="G18" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="H18" s="99" t="s">
+        <v>151</v>
+      </c>
+      <c r="I18" s="61" t="s">
+        <v>217</v>
+      </c>
+      <c r="J18" s="52" t="s">
+        <v>182</v>
+      </c>
+      <c r="K18" s="55">
         <v>1</v>
       </c>
-      <c r="L18" s="30">
+      <c r="L18" s="31">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M18" s="30">
-        <v>20</v>
-      </c>
-      <c r="N18" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O18" s="34">
-        <v>3.0300000000000001E-2</v>
-      </c>
-      <c r="P18" s="34">
+      <c r="M18" s="31">
+        <v>100</v>
+      </c>
+      <c r="N18" s="70" t="s">
+        <v>209</v>
+      </c>
+      <c r="O18" s="35">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="P18" s="35">
         <f t="shared" si="2"/>
-        <v>0.60599999999999998</v>
-      </c>
-      <c r="Q18" s="34"/>
-      <c r="R18" s="34"/>
+        <v>0.16</v>
+      </c>
+      <c r="Q18" s="35"/>
+      <c r="R18" s="35"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
@@ -2899,52 +2900,52 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="52" t="s">
-        <v>20</v>
-      </c>
-      <c r="D19" s="61" t="s">
-        <v>66</v>
-      </c>
-      <c r="E19" s="52" t="s">
-        <v>214</v>
-      </c>
-      <c r="F19" s="61" t="s">
-        <v>103</v>
-      </c>
-      <c r="G19" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H19" s="107" t="s">
-        <v>165</v>
-      </c>
-      <c r="I19" s="61" t="s">
-        <v>236</v>
-      </c>
-      <c r="J19" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="K19" s="55">
+      <c r="C19" s="53" t="s">
+        <v>15</v>
+      </c>
+      <c r="D19" s="62" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" s="53" t="s">
+        <v>91</v>
+      </c>
+      <c r="F19" s="62" t="s">
+        <v>129</v>
+      </c>
+      <c r="G19" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="H19" s="100" t="s">
+        <v>149</v>
+      </c>
+      <c r="I19" s="62" t="s">
+        <v>220</v>
+      </c>
+      <c r="J19" s="53" t="s">
+        <v>183</v>
+      </c>
+      <c r="K19" s="56">
         <v>1</v>
       </c>
-      <c r="L19" s="31">
+      <c r="L19" s="30">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M19" s="31">
-        <v>10</v>
-      </c>
-      <c r="N19" s="70" t="s">
-        <v>224</v>
-      </c>
-      <c r="O19" s="35">
-        <v>9.2899999999999996E-2</v>
-      </c>
-      <c r="P19" s="35">
+      <c r="M19" s="30">
+        <v>20</v>
+      </c>
+      <c r="N19" s="71" t="s">
+        <v>209</v>
+      </c>
+      <c r="O19" s="34">
+        <v>3.0300000000000001E-2</v>
+      </c>
+      <c r="P19" s="34">
         <f t="shared" si="2"/>
-        <v>0.92899999999999994</v>
-      </c>
-      <c r="Q19" s="35"/>
-      <c r="R19" s="35"/>
+        <v>0.60599999999999998</v>
+      </c>
+      <c r="Q19" s="34"/>
+      <c r="R19" s="34"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
@@ -2952,52 +2953,52 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="53" t="s">
-        <v>21</v>
-      </c>
-      <c r="D20" s="62" t="s">
-        <v>67</v>
-      </c>
-      <c r="E20" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="F20" s="62" t="s">
-        <v>104</v>
-      </c>
-      <c r="G20" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H20" s="108" t="s">
-        <v>166</v>
-      </c>
-      <c r="I20" s="62" t="s">
-        <v>237</v>
-      </c>
-      <c r="J20" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="K20" s="56">
+      <c r="C20" s="52" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="61" t="s">
+        <v>58</v>
+      </c>
+      <c r="E20" s="52" t="s">
+        <v>199</v>
+      </c>
+      <c r="F20" s="61" t="s">
+        <v>93</v>
+      </c>
+      <c r="G20" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="H20" s="99" t="s">
+        <v>153</v>
+      </c>
+      <c r="I20" s="61" t="s">
+        <v>221</v>
+      </c>
+      <c r="J20" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="K20" s="55">
         <v>1</v>
       </c>
-      <c r="L20" s="30">
+      <c r="L20" s="31">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M20" s="30">
-        <v>6</v>
-      </c>
-      <c r="N20" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O20" s="34">
-        <v>2.3371</v>
-      </c>
-      <c r="P20" s="34">
+      <c r="M20" s="31">
+        <v>10</v>
+      </c>
+      <c r="N20" s="70" t="s">
+        <v>209</v>
+      </c>
+      <c r="O20" s="35">
+        <v>9.2899999999999996E-2</v>
+      </c>
+      <c r="P20" s="35">
         <f t="shared" si="2"/>
-        <v>14.022600000000001</v>
-      </c>
-      <c r="Q20" s="34"/>
-      <c r="R20" s="34"/>
+        <v>0.92899999999999994</v>
+      </c>
+      <c r="Q20" s="35"/>
+      <c r="R20" s="35"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" s="1"/>
@@ -3005,158 +3006,158 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="52" t="s">
-        <v>22</v>
-      </c>
-      <c r="D21" s="61" t="s">
-        <v>68</v>
-      </c>
-      <c r="E21" s="52" t="s">
-        <v>214</v>
-      </c>
-      <c r="F21" s="61" t="s">
-        <v>105</v>
-      </c>
-      <c r="G21" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H21" s="107" t="s">
-        <v>167</v>
-      </c>
-      <c r="I21" s="61" t="s">
-        <v>238</v>
-      </c>
-      <c r="J21" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="K21" s="55">
+      <c r="C21" s="53" t="s">
+        <v>17</v>
+      </c>
+      <c r="D21" s="62" t="s">
+        <v>59</v>
+      </c>
+      <c r="E21" s="53" t="s">
+        <v>199</v>
+      </c>
+      <c r="F21" s="62" t="s">
+        <v>94</v>
+      </c>
+      <c r="G21" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="H21" s="100" t="s">
+        <v>154</v>
+      </c>
+      <c r="I21" s="62" t="s">
+        <v>222</v>
+      </c>
+      <c r="J21" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="K21" s="56">
         <v>1</v>
       </c>
-      <c r="L21" s="31">
+      <c r="L21" s="30">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M21" s="31">
-        <v>20</v>
-      </c>
-      <c r="N21" s="70" t="s">
-        <v>224</v>
-      </c>
-      <c r="O21" s="35">
-        <v>4.8399999999999999E-2</v>
-      </c>
-      <c r="P21" s="35">
+      <c r="M21" s="30">
+        <v>6</v>
+      </c>
+      <c r="N21" s="71" t="s">
+        <v>209</v>
+      </c>
+      <c r="O21" s="34">
+        <v>2.3371</v>
+      </c>
+      <c r="P21" s="34">
         <f t="shared" si="2"/>
-        <v>0.96799999999999997</v>
-      </c>
-      <c r="Q21" s="35"/>
-      <c r="R21" s="35"/>
-    </row>
-    <row r="22" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
+        <v>14.022600000000001</v>
+      </c>
+      <c r="Q21" s="34"/>
+      <c r="R21" s="34"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
       <c r="B22" s="78">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="53" t="s">
-        <v>23</v>
-      </c>
-      <c r="D22" s="62" t="s">
-        <v>69</v>
-      </c>
-      <c r="E22" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="F22" s="62" t="s">
-        <v>106</v>
-      </c>
-      <c r="G22" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H22" s="108" t="s">
-        <v>168</v>
-      </c>
-      <c r="I22" s="62" t="s">
-        <v>239</v>
-      </c>
-      <c r="J22" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="K22" s="56">
+      <c r="C22" s="52" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="61" t="s">
+        <v>60</v>
+      </c>
+      <c r="E22" s="52" t="s">
+        <v>199</v>
+      </c>
+      <c r="F22" s="61" t="s">
+        <v>95</v>
+      </c>
+      <c r="G22" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="H22" s="99" t="s">
+        <v>155</v>
+      </c>
+      <c r="I22" s="61" t="s">
+        <v>223</v>
+      </c>
+      <c r="J22" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="K22" s="55">
         <v>1</v>
       </c>
-      <c r="L22" s="30">
+      <c r="L22" s="31">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M22" s="30">
-        <v>6</v>
-      </c>
-      <c r="N22" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O22" s="34">
-        <v>0.18659999999999999</v>
-      </c>
-      <c r="P22" s="34">
+      <c r="M22" s="31">
+        <v>20</v>
+      </c>
+      <c r="N22" s="70" t="s">
+        <v>209</v>
+      </c>
+      <c r="O22" s="35">
+        <v>4.8399999999999999E-2</v>
+      </c>
+      <c r="P22" s="35">
         <f t="shared" si="2"/>
-        <v>1.1195999999999999</v>
-      </c>
-      <c r="Q22" s="34"/>
-      <c r="R22" s="34"/>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
+        <v>0.96799999999999997</v>
+      </c>
+      <c r="Q22" s="35"/>
+      <c r="R22" s="35"/>
+    </row>
+    <row r="23" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="78">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="52" t="s">
-        <v>24</v>
-      </c>
-      <c r="D23" s="105" t="s">
-        <v>280</v>
-      </c>
-      <c r="E23" s="52" t="s">
-        <v>107</v>
-      </c>
-      <c r="F23" s="63" t="s">
-        <v>281</v>
-      </c>
-      <c r="G23" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H23" s="107" t="s">
-        <v>282</v>
-      </c>
-      <c r="I23" s="61" t="s">
-        <v>285</v>
-      </c>
-      <c r="J23" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="K23" s="55">
+      <c r="C23" s="53" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" s="62" t="s">
+        <v>61</v>
+      </c>
+      <c r="E23" s="53" t="s">
+        <v>199</v>
+      </c>
+      <c r="F23" s="62" t="s">
+        <v>96</v>
+      </c>
+      <c r="G23" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="H23" s="100" t="s">
+        <v>156</v>
+      </c>
+      <c r="I23" s="62" t="s">
+        <v>224</v>
+      </c>
+      <c r="J23" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="K23" s="56">
         <v>1</v>
       </c>
-      <c r="L23" s="31">
+      <c r="L23" s="30">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M23" s="31">
-        <v>10</v>
-      </c>
-      <c r="N23" s="79" t="s">
-        <v>224</v>
-      </c>
-      <c r="O23" s="35">
-        <v>4.3099999999999999E-2</v>
-      </c>
-      <c r="P23" s="35">
+      <c r="M23" s="30">
+        <v>6</v>
+      </c>
+      <c r="N23" s="71" t="s">
+        <v>209</v>
+      </c>
+      <c r="O23" s="34">
+        <v>0.18659999999999999</v>
+      </c>
+      <c r="P23" s="34">
         <f t="shared" si="2"/>
-        <v>0.43099999999999999</v>
-      </c>
-      <c r="Q23" s="35"/>
-      <c r="R23" s="35"/>
+        <v>1.1195999999999999</v>
+      </c>
+      <c r="Q23" s="34"/>
+      <c r="R23" s="34"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
@@ -3164,52 +3165,52 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="53" t="s">
-        <v>25</v>
-      </c>
-      <c r="D24" s="62" t="s">
-        <v>70</v>
-      </c>
-      <c r="E24" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="F24" s="62" t="s">
-        <v>108</v>
-      </c>
-      <c r="G24" s="59" t="s">
-        <v>276</v>
-      </c>
-      <c r="H24" s="108" t="s">
-        <v>165</v>
-      </c>
-      <c r="I24" s="62" t="s">
-        <v>240</v>
-      </c>
-      <c r="J24" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="K24" s="56">
+      <c r="C24" s="52" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="97" t="s">
+        <v>263</v>
+      </c>
+      <c r="E24" s="52" t="s">
+        <v>97</v>
+      </c>
+      <c r="F24" s="63" t="s">
+        <v>264</v>
+      </c>
+      <c r="G24" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="H24" s="99" t="s">
+        <v>265</v>
+      </c>
+      <c r="I24" s="61" t="s">
+        <v>268</v>
+      </c>
+      <c r="J24" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="K24" s="55">
         <v>1</v>
       </c>
-      <c r="L24" s="30">
+      <c r="L24" s="31">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M24" s="30">
-        <v>6</v>
-      </c>
-      <c r="N24" s="72" t="s">
-        <v>224</v>
-      </c>
-      <c r="O24" s="37">
-        <v>0.1832</v>
-      </c>
-      <c r="P24" s="34">
+      <c r="M24" s="31">
+        <v>10</v>
+      </c>
+      <c r="N24" s="79" t="s">
+        <v>209</v>
+      </c>
+      <c r="O24" s="35">
+        <v>4.3099999999999999E-2</v>
+      </c>
+      <c r="P24" s="35">
         <f t="shared" si="2"/>
-        <v>1.0992</v>
-      </c>
-      <c r="Q24" s="34"/>
-      <c r="R24" s="34"/>
+        <v>0.43099999999999999</v>
+      </c>
+      <c r="Q24" s="35"/>
+      <c r="R24" s="35"/>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
@@ -3217,52 +3218,52 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="52" t="s">
-        <v>26</v>
-      </c>
-      <c r="D25" s="63" t="s">
-        <v>283</v>
-      </c>
-      <c r="E25" s="52" t="s">
-        <v>109</v>
-      </c>
-      <c r="F25" s="63" t="s">
-        <v>284</v>
-      </c>
-      <c r="G25" s="58" t="s">
-        <v>275</v>
-      </c>
-      <c r="H25" s="107" t="s">
-        <v>282</v>
-      </c>
-      <c r="I25" s="61" t="s">
-        <v>286</v>
-      </c>
-      <c r="J25" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="K25" s="55">
+      <c r="C25" s="53" t="s">
+        <v>21</v>
+      </c>
+      <c r="D25" s="62" t="s">
+        <v>62</v>
+      </c>
+      <c r="E25" s="53" t="s">
+        <v>199</v>
+      </c>
+      <c r="F25" s="62" t="s">
+        <v>98</v>
+      </c>
+      <c r="G25" s="59" t="s">
+        <v>259</v>
+      </c>
+      <c r="H25" s="100" t="s">
+        <v>153</v>
+      </c>
+      <c r="I25" s="62" t="s">
+        <v>225</v>
+      </c>
+      <c r="J25" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="K25" s="56">
         <v>1</v>
       </c>
-      <c r="L25" s="31">
+      <c r="L25" s="30">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M25" s="31">
-        <v>20</v>
-      </c>
-      <c r="N25" s="79" t="s">
-        <v>224</v>
-      </c>
-      <c r="O25" s="35">
-        <v>2.29E-2</v>
-      </c>
-      <c r="P25" s="35">
+      <c r="M25" s="30">
+        <v>6</v>
+      </c>
+      <c r="N25" s="72" t="s">
+        <v>209</v>
+      </c>
+      <c r="O25" s="37">
+        <v>0.1832</v>
+      </c>
+      <c r="P25" s="34">
         <f t="shared" si="2"/>
-        <v>0.45800000000000002</v>
-      </c>
-      <c r="Q25" s="35"/>
-      <c r="R25" s="35"/>
+        <v>1.0992</v>
+      </c>
+      <c r="Q25" s="34"/>
+      <c r="R25" s="34"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" s="1"/>
@@ -3270,50 +3271,52 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="88" t="s">
-        <v>27</v>
-      </c>
-      <c r="D26" s="89" t="s">
-        <v>71</v>
-      </c>
-      <c r="E26" s="88" t="s">
-        <v>214</v>
-      </c>
-      <c r="F26" s="89" t="s">
-        <v>110</v>
-      </c>
-      <c r="G26" s="96" t="s">
-        <v>275</v>
-      </c>
-      <c r="H26" s="109" t="s">
-        <v>164</v>
-      </c>
-      <c r="I26" s="90" t="s">
-        <v>275</v>
-      </c>
-      <c r="J26" s="88" t="s">
-        <v>198</v>
-      </c>
-      <c r="K26" s="91">
+      <c r="C26" s="52" t="s">
+        <v>22</v>
+      </c>
+      <c r="D26" s="63" t="s">
+        <v>266</v>
+      </c>
+      <c r="E26" s="52" t="s">
+        <v>99</v>
+      </c>
+      <c r="F26" s="63" t="s">
+        <v>267</v>
+      </c>
+      <c r="G26" s="58" t="s">
+        <v>258</v>
+      </c>
+      <c r="H26" s="99" t="s">
+        <v>265</v>
+      </c>
+      <c r="I26" s="61" t="s">
+        <v>269</v>
+      </c>
+      <c r="J26" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="K26" s="55">
         <v>1</v>
       </c>
-      <c r="L26" s="92">
+      <c r="L26" s="31">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M26" s="92">
-        <v>7</v>
-      </c>
-      <c r="N26" s="93"/>
-      <c r="O26" s="94"/>
-      <c r="P26" s="94">
+      <c r="M26" s="31">
+        <v>20</v>
+      </c>
+      <c r="N26" s="79" t="s">
+        <v>209</v>
+      </c>
+      <c r="O26" s="35">
+        <v>2.29E-2</v>
+      </c>
+      <c r="P26" s="35">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q26" s="95" t="s">
-        <v>294</v>
-      </c>
-      <c r="R26" s="94"/>
+        <v>0.45800000000000002</v>
+      </c>
+      <c r="Q26" s="35"/>
+      <c r="R26" s="35"/>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" s="1"/>
@@ -3321,52 +3324,50 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="52" t="s">
-        <v>28</v>
-      </c>
-      <c r="D27" s="61" t="s">
-        <v>72</v>
-      </c>
-      <c r="E27" s="52" t="s">
-        <v>214</v>
-      </c>
-      <c r="F27" s="61" t="s">
-        <v>111</v>
-      </c>
-      <c r="G27" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H27" s="107" t="s">
-        <v>169</v>
-      </c>
-      <c r="I27" s="61" t="s">
-        <v>241</v>
-      </c>
-      <c r="J27" s="52" t="s">
+      <c r="C27" s="88" t="s">
+        <v>23</v>
+      </c>
+      <c r="D27" s="89" t="s">
+        <v>63</v>
+      </c>
+      <c r="E27" s="88" t="s">
         <v>199</v>
       </c>
-      <c r="K27" s="55">
+      <c r="F27" s="89" t="s">
+        <v>100</v>
+      </c>
+      <c r="G27" s="96" t="s">
+        <v>258</v>
+      </c>
+      <c r="H27" s="101" t="s">
+        <v>152</v>
+      </c>
+      <c r="I27" s="90" t="s">
+        <v>258</v>
+      </c>
+      <c r="J27" s="88" t="s">
+        <v>184</v>
+      </c>
+      <c r="K27" s="91">
         <v>1</v>
       </c>
-      <c r="L27" s="31">
+      <c r="L27" s="92">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M27" s="31">
+      <c r="M27" s="92">
         <v>7</v>
       </c>
-      <c r="N27" s="70" t="s">
-        <v>224</v>
-      </c>
-      <c r="O27" s="35">
-        <v>0.1575</v>
-      </c>
-      <c r="P27" s="35">
+      <c r="N27" s="93"/>
+      <c r="O27" s="94"/>
+      <c r="P27" s="94">
         <f t="shared" si="2"/>
-        <v>1.1025</v>
-      </c>
-      <c r="Q27" s="35"/>
-      <c r="R27" s="35"/>
+        <v>0</v>
+      </c>
+      <c r="Q27" s="95" t="s">
+        <v>277</v>
+      </c>
+      <c r="R27" s="94"/>
     </row>
     <row r="28" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
@@ -3375,28 +3376,28 @@
         <v>19</v>
       </c>
       <c r="C28" s="53" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D28" s="62" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="E28" s="53" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="F28" s="62" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="G28" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H28" s="108" t="s">
-        <v>170</v>
+        <v>200</v>
+      </c>
+      <c r="H28" s="100" t="s">
+        <v>157</v>
       </c>
       <c r="I28" s="62" t="s">
-        <v>242</v>
+        <v>226</v>
       </c>
       <c r="J28" s="53" t="s">
-        <v>199</v>
+        <v>185</v>
       </c>
       <c r="K28" s="56">
         <v>1</v>
@@ -3409,7 +3410,7 @@
         <v>10</v>
       </c>
       <c r="N28" s="72" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O28" s="37">
         <v>4.5699999999999998E-2</v>
@@ -3428,28 +3429,28 @@
         <v>20</v>
       </c>
       <c r="C29" s="52" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="D29" s="61" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="E29" s="52" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="F29" s="61" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="G29" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H29" s="107" t="s">
-        <v>171</v>
+        <v>200</v>
+      </c>
+      <c r="H29" s="99" t="s">
+        <v>158</v>
       </c>
       <c r="I29" s="61" t="s">
-        <v>243</v>
+        <v>227</v>
       </c>
       <c r="J29" s="52" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="K29" s="55">
         <v>1</v>
@@ -3462,7 +3463,7 @@
         <v>10</v>
       </c>
       <c r="N29" s="70" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O29" s="35">
         <v>5.7299999999999997E-2</v>
@@ -3481,28 +3482,28 @@
         <v>21</v>
       </c>
       <c r="C30" s="53" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D30" s="62" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="E30" s="53" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="F30" s="62" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="G30" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H30" s="108" t="s">
-        <v>161</v>
+        <v>200</v>
+      </c>
+      <c r="H30" s="100" t="s">
+        <v>149</v>
       </c>
       <c r="I30" s="62" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="J30" s="53" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="K30" s="56">
         <v>1</v>
@@ -3515,7 +3516,7 @@
         <v>10</v>
       </c>
       <c r="N30" s="71" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O30" s="34">
         <v>6.4600000000000005E-2</v>
@@ -3534,28 +3535,28 @@
         <v>22</v>
       </c>
       <c r="C31" s="52" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D31" s="61" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="E31" s="52" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="F31" s="61" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="G31" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H31" s="107" t="s">
-        <v>161</v>
+        <v>200</v>
+      </c>
+      <c r="H31" s="99" t="s">
+        <v>149</v>
       </c>
       <c r="I31" s="61" t="s">
-        <v>246</v>
+        <v>230</v>
       </c>
       <c r="J31" s="58" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="K31" s="55">
         <v>1</v>
@@ -3568,7 +3569,7 @@
         <v>50</v>
       </c>
       <c r="N31" s="70" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O31" s="35">
         <v>8.6E-3</v>
@@ -3587,26 +3588,26 @@
         <v>23</v>
       </c>
       <c r="C32" s="53" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D32" s="62" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="E32" s="53" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="F32" s="62" t="s">
-        <v>115</v>
+        <v>104</v>
       </c>
       <c r="G32" s="53"/>
-      <c r="H32" s="108" t="s">
-        <v>172</v>
+      <c r="H32" s="100" t="s">
+        <v>159</v>
       </c>
       <c r="I32" s="62" t="s">
-        <v>244</v>
+        <v>228</v>
       </c>
       <c r="J32" s="53" t="s">
-        <v>202</v>
+        <v>188</v>
       </c>
       <c r="K32" s="56">
         <v>1</v>
@@ -3619,7 +3620,7 @@
         <v>10</v>
       </c>
       <c r="N32" s="72" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O32" s="37">
         <v>9.4299999999999995E-2</v>
@@ -3638,28 +3639,28 @@
         <v>24</v>
       </c>
       <c r="C33" s="52" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="D33" s="61" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="E33" s="52" t="s">
-        <v>116</v>
-      </c>
-      <c r="F33" s="116" t="s">
-        <v>144</v>
+        <v>105</v>
+      </c>
+      <c r="F33" s="108" t="s">
+        <v>133</v>
       </c>
       <c r="G33" s="52" t="s">
-        <v>247</v>
-      </c>
-      <c r="H33" s="107" t="s">
-        <v>173</v>
+        <v>231</v>
+      </c>
+      <c r="H33" s="99" t="s">
+        <v>160</v>
       </c>
       <c r="I33" s="61" t="s">
-        <v>248</v>
+        <v>232</v>
       </c>
       <c r="J33" s="58" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="K33" s="55">
         <v>2</v>
@@ -3672,7 +3673,7 @@
         <v>50</v>
       </c>
       <c r="N33" s="70" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O33" s="35">
         <v>1.7500000000000002E-2</v>
@@ -3691,28 +3692,28 @@
         <v>25</v>
       </c>
       <c r="C34" s="53" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="D34" s="62" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E34" s="53" t="s">
-        <v>116</v>
-      </c>
-      <c r="F34" s="117" t="s">
-        <v>145</v>
+        <v>105</v>
+      </c>
+      <c r="F34" s="109" t="s">
+        <v>134</v>
       </c>
       <c r="G34" s="53" t="s">
-        <v>249</v>
-      </c>
-      <c r="H34" s="108" t="s">
-        <v>173</v>
+        <v>233</v>
+      </c>
+      <c r="H34" s="100" t="s">
+        <v>160</v>
       </c>
       <c r="I34" s="62" t="s">
-        <v>250</v>
+        <v>234</v>
       </c>
       <c r="J34" s="59" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="K34" s="56">
         <v>1</v>
@@ -3725,7 +3726,7 @@
         <v>10</v>
       </c>
       <c r="N34" s="71" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O34" s="34">
         <v>5.2400000000000002E-2</v>
@@ -3744,28 +3745,28 @@
         <v>26</v>
       </c>
       <c r="C35" s="52" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="D35" s="61" t="s">
-        <v>287</v>
+        <v>270</v>
       </c>
       <c r="E35" s="52" t="s">
-        <v>288</v>
+        <v>271</v>
       </c>
       <c r="F35" s="61" t="s">
-        <v>289</v>
+        <v>272</v>
       </c>
       <c r="G35" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H35" s="110" t="s">
-        <v>290</v>
+        <v>200</v>
+      </c>
+      <c r="H35" s="102" t="s">
+        <v>273</v>
       </c>
       <c r="I35" s="61" t="s">
-        <v>291</v>
+        <v>274</v>
       </c>
       <c r="J35" s="52" t="s">
-        <v>203</v>
+        <v>189</v>
       </c>
       <c r="K35" s="55">
         <v>1</v>
@@ -3778,7 +3779,7 @@
         <v>50</v>
       </c>
       <c r="N35" s="79" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O35" s="35">
         <v>1.0500000000000001E-2</v>
@@ -3797,28 +3798,28 @@
         <v>27</v>
       </c>
       <c r="C36" s="53" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D36" s="62" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="E36" s="53" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="F36" s="62" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="G36" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H36" s="108" t="s">
-        <v>163</v>
+        <v>200</v>
+      </c>
+      <c r="H36" s="100" t="s">
+        <v>151</v>
       </c>
       <c r="I36" s="62" t="s">
-        <v>269</v>
+        <v>252</v>
       </c>
       <c r="J36" s="53" t="s">
-        <v>204</v>
+        <v>190</v>
       </c>
       <c r="K36" s="56">
         <v>4</v>
@@ -3831,7 +3832,7 @@
         <v>100</v>
       </c>
       <c r="N36" s="71" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O36" s="34">
         <v>5.9999999999999995E-4</v>
@@ -3850,28 +3851,28 @@
         <v>28</v>
       </c>
       <c r="C37" s="52" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D37" s="61" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="E37" s="52" t="s">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="F37" s="61" t="s">
-        <v>146</v>
+        <v>135</v>
       </c>
       <c r="G37" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H37" s="107" t="s">
-        <v>163</v>
+        <v>200</v>
+      </c>
+      <c r="H37" s="99" t="s">
+        <v>151</v>
       </c>
       <c r="I37" s="61" t="s">
-        <v>251</v>
+        <v>235</v>
       </c>
       <c r="J37" s="52" t="s">
-        <v>205</v>
+        <v>191</v>
       </c>
       <c r="K37" s="55">
         <v>10</v>
@@ -3884,7 +3885,7 @@
         <v>100</v>
       </c>
       <c r="N37" s="70" t="s">
-        <v>224</v>
+        <v>209</v>
       </c>
       <c r="O37" s="35">
         <v>6.9999999999999999E-4</v>
@@ -3896,58 +3897,58 @@
       <c r="Q37" s="35"/>
       <c r="R37" s="35"/>
     </row>
-    <row r="38" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
       <c r="B38" s="78">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="D38" s="62" t="s">
-        <v>81</v>
-      </c>
-      <c r="E38" s="53" t="s">
-        <v>118</v>
-      </c>
-      <c r="F38" s="62" t="s">
-        <v>147</v>
-      </c>
-      <c r="G38" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H38" s="108" t="s">
-        <v>174</v>
-      </c>
-      <c r="I38" s="62" t="s">
-        <v>252</v>
-      </c>
-      <c r="J38" s="53" t="s">
-        <v>206</v>
-      </c>
-      <c r="K38" s="56">
-        <v>1</v>
-      </c>
-      <c r="L38" s="30">
+      <c r="C38" s="52" t="s">
+        <v>287</v>
+      </c>
+      <c r="D38" s="61" t="s">
+        <v>72</v>
+      </c>
+      <c r="E38" s="52" t="s">
+        <v>107</v>
+      </c>
+      <c r="F38" s="108" t="s">
+        <v>136</v>
+      </c>
+      <c r="G38" s="52" t="s">
+        <v>237</v>
+      </c>
+      <c r="H38" s="99" t="s">
+        <v>161</v>
+      </c>
+      <c r="I38" s="61" t="s">
+        <v>238</v>
+      </c>
+      <c r="J38" s="52" t="s">
+        <v>192</v>
+      </c>
+      <c r="K38" s="55">
+        <v>8</v>
+      </c>
+      <c r="L38" s="31">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="M38" s="30">
+        <v>40</v>
+      </c>
+      <c r="M38" s="31">
         <v>100</v>
       </c>
-      <c r="N38" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O38" s="34">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="P38" s="34">
+      <c r="N38" s="70" t="s">
+        <v>209</v>
+      </c>
+      <c r="O38" s="35">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="P38" s="35">
         <f t="shared" si="2"/>
-        <v>0.05</v>
-      </c>
-      <c r="Q38" s="34"/>
-      <c r="R38" s="34"/>
+        <v>0.06</v>
+      </c>
+      <c r="Q38" s="35"/>
+      <c r="R38" s="35"/>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" s="1"/>
@@ -3955,52 +3956,52 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="52" t="s">
-        <v>40</v>
-      </c>
-      <c r="D39" s="61" t="s">
-        <v>82</v>
-      </c>
-      <c r="E39" s="52" t="s">
-        <v>118</v>
-      </c>
-      <c r="F39" s="116" t="s">
-        <v>148</v>
-      </c>
-      <c r="G39" s="52" t="s">
-        <v>254</v>
-      </c>
-      <c r="H39" s="107" t="s">
-        <v>175</v>
-      </c>
-      <c r="I39" s="61" t="s">
-        <v>255</v>
-      </c>
-      <c r="J39" s="52" t="s">
-        <v>207</v>
-      </c>
-      <c r="K39" s="55">
-        <v>7</v>
-      </c>
-      <c r="L39" s="31">
+      <c r="C39" s="53" t="s">
+        <v>34</v>
+      </c>
+      <c r="D39" s="62" t="s">
+        <v>73</v>
+      </c>
+      <c r="E39" s="53" t="s">
+        <v>107</v>
+      </c>
+      <c r="F39" s="109" t="s">
+        <v>137</v>
+      </c>
+      <c r="G39" s="53" t="s">
+        <v>239</v>
+      </c>
+      <c r="H39" s="100" t="s">
+        <v>161</v>
+      </c>
+      <c r="I39" s="62" t="s">
+        <v>240</v>
+      </c>
+      <c r="J39" s="53" t="s">
+        <v>193</v>
+      </c>
+      <c r="K39" s="56">
+        <v>2</v>
+      </c>
+      <c r="L39" s="30">
         <f t="shared" si="1"/>
-        <v>35</v>
-      </c>
-      <c r="M39" s="31">
+        <v>10</v>
+      </c>
+      <c r="M39" s="30">
         <v>100</v>
       </c>
-      <c r="N39" s="70" t="s">
-        <v>224</v>
-      </c>
-      <c r="O39" s="35">
-        <v>5.9999999999999995E-4</v>
-      </c>
-      <c r="P39" s="35">
+      <c r="N39" s="71" t="s">
+        <v>209</v>
+      </c>
+      <c r="O39" s="34">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="P39" s="34">
         <f t="shared" si="2"/>
-        <v>0.06</v>
-      </c>
-      <c r="Q39" s="35"/>
-      <c r="R39" s="35"/>
+        <v>0.08</v>
+      </c>
+      <c r="Q39" s="34"/>
+      <c r="R39" s="34"/>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" s="1"/>
@@ -4008,52 +4009,52 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C40" s="53" t="s">
-        <v>41</v>
-      </c>
-      <c r="D40" s="62" t="s">
-        <v>83</v>
-      </c>
-      <c r="E40" s="53" t="s">
-        <v>118</v>
-      </c>
-      <c r="F40" s="117" t="s">
-        <v>149</v>
-      </c>
-      <c r="G40" s="53" t="s">
-        <v>256</v>
-      </c>
-      <c r="H40" s="108" t="s">
-        <v>175</v>
-      </c>
-      <c r="I40" s="62" t="s">
-        <v>257</v>
-      </c>
-      <c r="J40" s="53" t="s">
-        <v>208</v>
-      </c>
-      <c r="K40" s="56">
+      <c r="C40" s="52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D40" s="61" t="s">
+        <v>74</v>
+      </c>
+      <c r="E40" s="52" t="s">
+        <v>106</v>
+      </c>
+      <c r="F40" s="108" t="s">
+        <v>138</v>
+      </c>
+      <c r="G40" s="52" t="s">
+        <v>241</v>
+      </c>
+      <c r="H40" s="99" t="s">
+        <v>162</v>
+      </c>
+      <c r="I40" s="61" t="s">
+        <v>242</v>
+      </c>
+      <c r="J40" s="52" t="s">
+        <v>194</v>
+      </c>
+      <c r="K40" s="55">
         <v>2</v>
       </c>
-      <c r="L40" s="30">
+      <c r="L40" s="31">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="M40" s="30">
+      <c r="M40" s="31">
         <v>100</v>
       </c>
-      <c r="N40" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O40" s="34">
-        <v>8.0000000000000004E-4</v>
-      </c>
-      <c r="P40" s="34">
+      <c r="N40" s="70" t="s">
+        <v>209</v>
+      </c>
+      <c r="O40" s="35">
+        <v>3.5999999999999999E-3</v>
+      </c>
+      <c r="P40" s="35">
         <f t="shared" si="2"/>
-        <v>0.08</v>
-      </c>
-      <c r="Q40" s="34"/>
-      <c r="R40" s="34"/>
+        <v>0.36</v>
+      </c>
+      <c r="Q40" s="35"/>
+      <c r="R40" s="35"/>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
@@ -4061,52 +4062,52 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C41" s="52" t="s">
-        <v>42</v>
-      </c>
-      <c r="D41" s="61" t="s">
-        <v>84</v>
-      </c>
-      <c r="E41" s="52" t="s">
-        <v>117</v>
-      </c>
-      <c r="F41" s="116" t="s">
-        <v>150</v>
-      </c>
-      <c r="G41" s="52" t="s">
-        <v>258</v>
-      </c>
-      <c r="H41" s="107" t="s">
-        <v>176</v>
-      </c>
-      <c r="I41" s="61" t="s">
-        <v>259</v>
-      </c>
-      <c r="J41" s="52" t="s">
+      <c r="C41" s="53" t="s">
+        <v>36</v>
+      </c>
+      <c r="D41" s="62" t="s">
+        <v>75</v>
+      </c>
+      <c r="E41" s="53" t="s">
+        <v>107</v>
+      </c>
+      <c r="F41" s="62" t="s">
+        <v>139</v>
+      </c>
+      <c r="G41" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="H41" s="100" t="s">
+        <v>151</v>
+      </c>
+      <c r="I41" s="62" t="s">
+        <v>236</v>
+      </c>
+      <c r="J41" s="53" t="s">
+        <v>195</v>
+      </c>
+      <c r="K41" s="56">
+        <v>1</v>
+      </c>
+      <c r="L41" s="30">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="M41" s="30">
+        <v>50</v>
+      </c>
+      <c r="N41" s="71" t="s">
         <v>209</v>
       </c>
-      <c r="K41" s="55">
-        <v>2</v>
-      </c>
-      <c r="L41" s="31">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="M41" s="31">
-        <v>100</v>
-      </c>
-      <c r="N41" s="70" t="s">
-        <v>224</v>
-      </c>
-      <c r="O41" s="35">
-        <v>3.5999999999999999E-3</v>
-      </c>
-      <c r="P41" s="35">
+      <c r="O41" s="34">
+        <v>6.9999999999999999E-4</v>
+      </c>
+      <c r="P41" s="34">
         <f t="shared" si="2"/>
-        <v>0.36</v>
-      </c>
-      <c r="Q41" s="35"/>
-      <c r="R41" s="35"/>
+        <v>3.4999999999999996E-2</v>
+      </c>
+      <c r="Q41" s="34"/>
+      <c r="R41" s="34"/>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" s="1"/>
@@ -4114,102 +4115,102 @@
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="C42" s="53" t="s">
-        <v>43</v>
-      </c>
-      <c r="D42" s="62" t="s">
-        <v>85</v>
-      </c>
-      <c r="E42" s="53" t="s">
-        <v>118</v>
-      </c>
-      <c r="F42" s="62" t="s">
-        <v>151</v>
-      </c>
-      <c r="G42" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H42" s="108" t="s">
-        <v>163</v>
-      </c>
-      <c r="I42" s="62" t="s">
-        <v>253</v>
-      </c>
-      <c r="J42" s="53" t="s">
-        <v>210</v>
-      </c>
-      <c r="K42" s="56">
-        <v>1</v>
-      </c>
-      <c r="L42" s="30">
+      <c r="C42" s="52" t="s">
+        <v>37</v>
+      </c>
+      <c r="D42" s="61" t="s">
+        <v>76</v>
+      </c>
+      <c r="E42" s="52" t="s">
+        <v>108</v>
+      </c>
+      <c r="F42" s="63" t="s">
+        <v>201</v>
+      </c>
+      <c r="G42" s="58"/>
+      <c r="H42" s="103" t="s">
+        <v>201</v>
+      </c>
+      <c r="I42" s="63" t="s">
+        <v>255</v>
+      </c>
+      <c r="J42" s="58" t="s">
+        <v>201</v>
+      </c>
+      <c r="K42" s="55">
+        <v>3</v>
+      </c>
+      <c r="L42" s="31">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="M42" s="30">
-        <v>50</v>
-      </c>
-      <c r="N42" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O42" s="34">
-        <v>6.9999999999999999E-4</v>
-      </c>
-      <c r="P42" s="34">
-        <f t="shared" si="2"/>
-        <v>3.4999999999999996E-2</v>
-      </c>
-      <c r="Q42" s="34"/>
-      <c r="R42" s="34"/>
-    </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="M42" s="65" t="s">
+        <v>200</v>
+      </c>
+      <c r="N42" s="65" t="s">
+        <v>201</v>
+      </c>
+      <c r="O42" s="65" t="s">
+        <v>200</v>
+      </c>
+      <c r="P42" s="65" t="s">
+        <v>201</v>
+      </c>
+      <c r="Q42" s="65"/>
+      <c r="R42" s="65"/>
+    </row>
+    <row r="43" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="78">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="52" t="s">
-        <v>44</v>
-      </c>
-      <c r="D43" s="61" t="s">
-        <v>86</v>
-      </c>
-      <c r="E43" s="52" t="s">
-        <v>119</v>
-      </c>
-      <c r="F43" s="63" t="s">
-        <v>216</v>
-      </c>
-      <c r="G43" s="58"/>
-      <c r="H43" s="111" t="s">
-        <v>216</v>
-      </c>
-      <c r="I43" s="63" t="s">
-        <v>272</v>
-      </c>
-      <c r="J43" s="58" t="s">
-        <v>216</v>
-      </c>
-      <c r="K43" s="55">
-        <v>3</v>
-      </c>
-      <c r="L43" s="31">
+      <c r="C43" s="53" t="s">
+        <v>288</v>
+      </c>
+      <c r="D43" s="62" t="s">
+        <v>77</v>
+      </c>
+      <c r="E43" s="53" t="s">
+        <v>199</v>
+      </c>
+      <c r="F43" s="62" t="s">
+        <v>109</v>
+      </c>
+      <c r="G43" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="H43" s="100" t="s">
+        <v>163</v>
+      </c>
+      <c r="I43" s="62" t="s">
+        <v>243</v>
+      </c>
+      <c r="J43" s="59" t="s">
+        <v>201</v>
+      </c>
+      <c r="K43" s="56">
+        <v>2</v>
+      </c>
+      <c r="L43" s="30">
         <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-      <c r="M43" s="65" t="s">
-        <v>215</v>
-      </c>
-      <c r="N43" s="65" t="s">
-        <v>216</v>
-      </c>
-      <c r="O43" s="65" t="s">
-        <v>215</v>
-      </c>
-      <c r="P43" s="65" t="s">
-        <v>216</v>
-      </c>
-      <c r="Q43" s="65"/>
-      <c r="R43" s="65"/>
+        <v>10</v>
+      </c>
+      <c r="M43" s="30">
+        <v>10</v>
+      </c>
+      <c r="N43" s="71" t="s">
+        <v>209</v>
+      </c>
+      <c r="O43" s="34">
+        <v>5.9900000000000002E-2</v>
+      </c>
+      <c r="P43" s="34">
+        <f t="shared" si="2"/>
+        <v>0.59899999999999998</v>
+      </c>
+      <c r="Q43" s="34"/>
+      <c r="R43" s="34"/>
     </row>
     <row r="44" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A44" s="1"/>
@@ -4217,156 +4218,152 @@
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="C44" s="53" t="s">
-        <v>45</v>
-      </c>
-      <c r="D44" s="62" t="s">
-        <v>87</v>
-      </c>
-      <c r="E44" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="F44" s="62" t="s">
-        <v>120</v>
-      </c>
-      <c r="G44" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H44" s="108" t="s">
-        <v>177</v>
-      </c>
-      <c r="I44" s="62" t="s">
-        <v>260</v>
-      </c>
-      <c r="J44" s="59" t="s">
-        <v>216</v>
-      </c>
-      <c r="K44" s="56">
+      <c r="C44" s="88" t="s">
+        <v>38</v>
+      </c>
+      <c r="D44" s="89" t="s">
+        <v>78</v>
+      </c>
+      <c r="E44" s="88" t="s">
+        <v>110</v>
+      </c>
+      <c r="F44" s="89" t="s">
+        <v>140</v>
+      </c>
+      <c r="G44" s="96" t="s">
+        <v>255</v>
+      </c>
+      <c r="H44" s="101" t="s">
+        <v>164</v>
+      </c>
+      <c r="I44" s="90" t="s">
+        <v>255</v>
+      </c>
+      <c r="J44" s="96" t="s">
+        <v>201</v>
+      </c>
+      <c r="K44" s="91">
         <v>1</v>
       </c>
-      <c r="L44" s="30">
+      <c r="L44" s="92">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M44" s="30">
-        <v>10</v>
-      </c>
-      <c r="N44" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O44" s="34">
-        <v>5.9900000000000002E-2</v>
-      </c>
-      <c r="P44" s="34">
+      <c r="M44" s="92">
+        <v>6</v>
+      </c>
+      <c r="N44" s="93"/>
+      <c r="O44" s="94"/>
+      <c r="P44" s="94">
         <f t="shared" si="2"/>
-        <v>0.59899999999999998</v>
-      </c>
-      <c r="Q44" s="34"/>
-      <c r="R44" s="34"/>
-    </row>
-    <row r="45" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="95" t="s">
+        <v>277</v>
+      </c>
+      <c r="R44" s="94"/>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
       <c r="B45" s="78">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C45" s="88" t="s">
-        <v>46</v>
-      </c>
-      <c r="D45" s="89" t="s">
-        <v>88</v>
-      </c>
-      <c r="E45" s="88" t="s">
-        <v>121</v>
-      </c>
-      <c r="F45" s="89" t="s">
-        <v>152</v>
-      </c>
-      <c r="G45" s="96" t="s">
-        <v>272</v>
-      </c>
-      <c r="H45" s="109" t="s">
-        <v>178</v>
-      </c>
-      <c r="I45" s="90" t="s">
-        <v>272</v>
-      </c>
-      <c r="J45" s="96" t="s">
-        <v>216</v>
-      </c>
-      <c r="K45" s="91">
+      <c r="C45" s="53" t="s">
+        <v>39</v>
+      </c>
+      <c r="D45" s="62" t="s">
+        <v>79</v>
+      </c>
+      <c r="E45" s="53" t="s">
+        <v>111</v>
+      </c>
+      <c r="F45" s="62" t="s">
+        <v>141</v>
+      </c>
+      <c r="G45" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="H45" s="100" t="s">
+        <v>165</v>
+      </c>
+      <c r="I45" s="62" t="s">
+        <v>244</v>
+      </c>
+      <c r="J45" s="59" t="s">
+        <v>201</v>
+      </c>
+      <c r="K45" s="56">
         <v>1</v>
       </c>
-      <c r="L45" s="92">
+      <c r="L45" s="30">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M45" s="92">
+      <c r="M45" s="30">
         <v>6</v>
       </c>
-      <c r="N45" s="93"/>
-      <c r="O45" s="94"/>
-      <c r="P45" s="94">
+      <c r="N45" s="71" t="s">
+        <v>209</v>
+      </c>
+      <c r="O45" s="34">
+        <v>0.49409999999999998</v>
+      </c>
+      <c r="P45" s="34">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q45" s="95" t="s">
-        <v>294</v>
-      </c>
-      <c r="R45" s="94"/>
-    </row>
-    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
+        <v>2.9645999999999999</v>
+      </c>
+      <c r="Q45" s="34"/>
+      <c r="R45" s="34"/>
+    </row>
+    <row r="46" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A46" s="1"/>
       <c r="B46" s="78">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="C46" s="53" t="s">
-        <v>47</v>
-      </c>
-      <c r="D46" s="62" t="s">
-        <v>89</v>
-      </c>
-      <c r="E46" s="53" t="s">
-        <v>122</v>
-      </c>
-      <c r="F46" s="62" t="s">
-        <v>153</v>
-      </c>
-      <c r="G46" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H46" s="108" t="s">
-        <v>179</v>
-      </c>
-      <c r="I46" s="62" t="s">
-        <v>261</v>
-      </c>
-      <c r="J46" s="59" t="s">
-        <v>216</v>
-      </c>
-      <c r="K46" s="56">
+      <c r="C46" s="88" t="s">
+        <v>40</v>
+      </c>
+      <c r="D46" s="89" t="s">
+        <v>80</v>
+      </c>
+      <c r="E46" s="88" t="s">
+        <v>112</v>
+      </c>
+      <c r="F46" s="89" t="s">
+        <v>142</v>
+      </c>
+      <c r="G46" s="96" t="s">
+        <v>200</v>
+      </c>
+      <c r="H46" s="101" t="s">
+        <v>166</v>
+      </c>
+      <c r="I46" s="90" t="s">
+        <v>255</v>
+      </c>
+      <c r="J46" s="96" t="s">
+        <v>201</v>
+      </c>
+      <c r="K46" s="91">
         <v>1</v>
       </c>
-      <c r="L46" s="30">
+      <c r="L46" s="92">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M46" s="30">
+      <c r="M46" s="92">
         <v>6</v>
       </c>
-      <c r="N46" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O46" s="34">
-        <v>0.49409999999999998</v>
-      </c>
-      <c r="P46" s="34">
+      <c r="N46" s="93"/>
+      <c r="O46" s="94"/>
+      <c r="P46" s="94">
         <f t="shared" si="2"/>
-        <v>2.9645999999999999</v>
-      </c>
-      <c r="Q46" s="34"/>
-      <c r="R46" s="34"/>
+        <v>0</v>
+      </c>
+      <c r="Q46" s="95"/>
+      <c r="R46" s="94"/>
     </row>
     <row r="47" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
@@ -4374,103 +4371,105 @@
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="C47" s="88" t="s">
-        <v>48</v>
-      </c>
-      <c r="D47" s="89" t="s">
-        <v>90</v>
-      </c>
-      <c r="E47" s="88" t="s">
-        <v>123</v>
-      </c>
-      <c r="F47" s="89" t="s">
-        <v>154</v>
-      </c>
-      <c r="G47" s="96" t="s">
-        <v>215</v>
-      </c>
-      <c r="H47" s="109" t="s">
-        <v>180</v>
-      </c>
-      <c r="I47" s="90" t="s">
-        <v>272</v>
-      </c>
-      <c r="J47" s="96" t="s">
-        <v>216</v>
-      </c>
-      <c r="K47" s="91">
+      <c r="C47" s="80" t="s">
+        <v>41</v>
+      </c>
+      <c r="D47" s="81" t="s">
+        <v>81</v>
+      </c>
+      <c r="E47" s="80" t="s">
+        <v>113</v>
+      </c>
+      <c r="F47" s="81" t="s">
+        <v>143</v>
+      </c>
+      <c r="G47" s="82" t="s">
+        <v>200</v>
+      </c>
+      <c r="H47" s="104" t="s">
+        <v>167</v>
+      </c>
+      <c r="I47" s="81" t="s">
+        <v>245</v>
+      </c>
+      <c r="J47" s="82" t="s">
+        <v>201</v>
+      </c>
+      <c r="K47" s="83">
         <v>1</v>
       </c>
-      <c r="L47" s="92">
+      <c r="L47" s="84">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M47" s="92">
+      <c r="M47" s="84">
         <v>6</v>
       </c>
-      <c r="N47" s="93"/>
-      <c r="O47" s="94"/>
-      <c r="P47" s="94">
+      <c r="N47" s="85" t="s">
+        <v>209</v>
+      </c>
+      <c r="O47" s="86">
+        <v>12.0892</v>
+      </c>
+      <c r="P47" s="86">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q47" s="95"/>
-      <c r="R47" s="94"/>
-    </row>
-    <row r="48" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
+        <v>72.535200000000003</v>
+      </c>
+      <c r="Q47" s="87" t="s">
+        <v>275</v>
+      </c>
+      <c r="R47" s="86"/>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
       <c r="B48" s="78">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="C48" s="80" t="s">
-        <v>49</v>
-      </c>
-      <c r="D48" s="81" t="s">
-        <v>91</v>
-      </c>
-      <c r="E48" s="80" t="s">
-        <v>124</v>
-      </c>
-      <c r="F48" s="81" t="s">
-        <v>155</v>
-      </c>
-      <c r="G48" s="82" t="s">
-        <v>215</v>
-      </c>
-      <c r="H48" s="112" t="s">
-        <v>181</v>
-      </c>
-      <c r="I48" s="81" t="s">
-        <v>262</v>
-      </c>
-      <c r="J48" s="82" t="s">
-        <v>216</v>
-      </c>
-      <c r="K48" s="83">
+      <c r="C48" s="88" t="s">
+        <v>42</v>
+      </c>
+      <c r="D48" s="89" t="s">
+        <v>82</v>
+      </c>
+      <c r="E48" s="88" t="s">
+        <v>114</v>
+      </c>
+      <c r="F48" s="89" t="s">
+        <v>144</v>
+      </c>
+      <c r="G48" s="96" t="s">
+        <v>200</v>
+      </c>
+      <c r="H48" s="101" t="s">
+        <v>168</v>
+      </c>
+      <c r="I48" s="90" t="s">
+        <v>200</v>
+      </c>
+      <c r="J48" s="96" t="s">
+        <v>201</v>
+      </c>
+      <c r="K48" s="91">
         <v>1</v>
       </c>
-      <c r="L48" s="84">
+      <c r="L48" s="92">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M48" s="84">
+      <c r="M48" s="92">
         <v>6</v>
       </c>
-      <c r="N48" s="85" t="s">
-        <v>224</v>
-      </c>
-      <c r="O48" s="86">
-        <v>12.0892</v>
-      </c>
-      <c r="P48" s="86">
+      <c r="N48" s="93"/>
+      <c r="O48" s="94"/>
+      <c r="P48" s="94">
         <f t="shared" si="2"/>
-        <v>72.535200000000003</v>
-      </c>
-      <c r="Q48" s="87" t="s">
-        <v>292</v>
-      </c>
-      <c r="R48" s="86"/>
+        <v>0</v>
+      </c>
+      <c r="Q48" s="95" t="s">
+        <v>277</v>
+      </c>
+      <c r="R48" s="94"/>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
@@ -4478,103 +4477,105 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="C49" s="88" t="s">
-        <v>50</v>
-      </c>
-      <c r="D49" s="89" t="s">
-        <v>92</v>
-      </c>
-      <c r="E49" s="88" t="s">
-        <v>125</v>
-      </c>
-      <c r="F49" s="89" t="s">
-        <v>156</v>
-      </c>
-      <c r="G49" s="96" t="s">
-        <v>215</v>
-      </c>
-      <c r="H49" s="109" t="s">
-        <v>182</v>
-      </c>
-      <c r="I49" s="90" t="s">
-        <v>215</v>
-      </c>
-      <c r="J49" s="96" t="s">
-        <v>216</v>
-      </c>
-      <c r="K49" s="91">
+      <c r="C49" s="53" t="s">
+        <v>43</v>
+      </c>
+      <c r="D49" s="62" t="s">
+        <v>83</v>
+      </c>
+      <c r="E49" s="53" t="s">
+        <v>115</v>
+      </c>
+      <c r="F49" s="62" t="s">
+        <v>145</v>
+      </c>
+      <c r="G49" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="H49" s="100" t="s">
+        <v>169</v>
+      </c>
+      <c r="I49" s="62" t="s">
+        <v>246</v>
+      </c>
+      <c r="J49" s="59" t="s">
+        <v>201</v>
+      </c>
+      <c r="K49" s="56">
         <v>1</v>
       </c>
-      <c r="L49" s="92">
+      <c r="L49" s="30">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M49" s="92">
+      <c r="M49" s="30">
         <v>6</v>
       </c>
-      <c r="N49" s="93"/>
-      <c r="O49" s="94"/>
-      <c r="P49" s="94">
+      <c r="N49" s="71" t="s">
+        <v>209</v>
+      </c>
+      <c r="O49" s="34">
+        <v>2.851</v>
+      </c>
+      <c r="P49" s="34">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q49" s="95" t="s">
-        <v>294</v>
-      </c>
-      <c r="R49" s="94"/>
-    </row>
-    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
+        <v>17.106000000000002</v>
+      </c>
+      <c r="Q49" s="34"/>
+      <c r="R49" s="34"/>
+    </row>
+    <row r="50" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A50" s="1"/>
       <c r="B50" s="78">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="C50" s="53" t="s">
-        <v>51</v>
-      </c>
-      <c r="D50" s="62" t="s">
-        <v>93</v>
-      </c>
-      <c r="E50" s="53" t="s">
-        <v>126</v>
-      </c>
-      <c r="F50" s="62" t="s">
-        <v>157</v>
-      </c>
-      <c r="G50" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H50" s="108" t="s">
-        <v>183</v>
-      </c>
-      <c r="I50" s="62" t="s">
-        <v>263</v>
-      </c>
-      <c r="J50" s="59" t="s">
-        <v>216</v>
-      </c>
-      <c r="K50" s="56">
+      <c r="C50" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="D50" s="61" t="s">
+        <v>84</v>
+      </c>
+      <c r="E50" s="52" t="s">
+        <v>116</v>
+      </c>
+      <c r="F50" s="61" t="s">
+        <v>146</v>
+      </c>
+      <c r="G50" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="H50" s="99" t="s">
+        <v>170</v>
+      </c>
+      <c r="I50" s="61" t="s">
+        <v>247</v>
+      </c>
+      <c r="J50" s="58" t="s">
+        <v>201</v>
+      </c>
+      <c r="K50" s="55">
         <v>1</v>
       </c>
-      <c r="L50" s="30">
+      <c r="L50" s="31">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M50" s="30">
+      <c r="M50" s="31">
         <v>6</v>
       </c>
-      <c r="N50" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O50" s="34">
-        <v>2.851</v>
-      </c>
-      <c r="P50" s="34">
+      <c r="N50" s="70" t="s">
+        <v>209</v>
+      </c>
+      <c r="O50" s="35">
+        <v>4.3278999999999996</v>
+      </c>
+      <c r="P50" s="35">
         <f t="shared" si="2"/>
-        <v>17.106000000000002</v>
-      </c>
-      <c r="Q50" s="34"/>
-      <c r="R50" s="34"/>
+        <v>25.967399999999998</v>
+      </c>
+      <c r="Q50" s="35"/>
+      <c r="R50" s="35"/>
     </row>
     <row r="51" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A51" s="1"/>
@@ -4582,52 +4583,52 @@
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="C51" s="52" t="s">
-        <v>52</v>
-      </c>
-      <c r="D51" s="61" t="s">
-        <v>94</v>
-      </c>
-      <c r="E51" s="52" t="s">
-        <v>127</v>
-      </c>
-      <c r="F51" s="61" t="s">
-        <v>158</v>
-      </c>
-      <c r="G51" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H51" s="107" t="s">
-        <v>184</v>
-      </c>
-      <c r="I51" s="61" t="s">
-        <v>264</v>
-      </c>
-      <c r="J51" s="58" t="s">
-        <v>216</v>
-      </c>
-      <c r="K51" s="55">
+      <c r="C51" s="53" t="s">
+        <v>45</v>
+      </c>
+      <c r="D51" s="62" t="s">
+        <v>85</v>
+      </c>
+      <c r="E51" s="53" t="s">
+        <v>117</v>
+      </c>
+      <c r="F51" s="62" t="s">
+        <v>147</v>
+      </c>
+      <c r="G51" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="H51" s="100" t="s">
+        <v>171</v>
+      </c>
+      <c r="I51" s="62" t="s">
+        <v>248</v>
+      </c>
+      <c r="J51" s="59" t="s">
+        <v>201</v>
+      </c>
+      <c r="K51" s="56">
         <v>1</v>
       </c>
-      <c r="L51" s="31">
+      <c r="L51" s="30">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M51" s="31">
-        <v>6</v>
-      </c>
-      <c r="N51" s="70" t="s">
-        <v>224</v>
-      </c>
-      <c r="O51" s="35">
-        <v>4.3278999999999996</v>
-      </c>
-      <c r="P51" s="35">
+      <c r="M51" s="30">
+        <v>10</v>
+      </c>
+      <c r="N51" s="71" t="s">
+        <v>209</v>
+      </c>
+      <c r="O51" s="34">
+        <v>2.0400000000000001E-2</v>
+      </c>
+      <c r="P51" s="34">
         <f t="shared" si="2"/>
-        <v>25.967399999999998</v>
-      </c>
-      <c r="Q51" s="35"/>
-      <c r="R51" s="35"/>
+        <v>0.20400000000000001</v>
+      </c>
+      <c r="Q51" s="34"/>
+      <c r="R51" s="34"/>
     </row>
     <row r="52" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A52" s="1"/>
@@ -4635,52 +4636,52 @@
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="C52" s="53" t="s">
-        <v>53</v>
-      </c>
-      <c r="D52" s="62" t="s">
-        <v>95</v>
-      </c>
-      <c r="E52" s="53" t="s">
-        <v>128</v>
-      </c>
-      <c r="F52" s="62" t="s">
-        <v>159</v>
-      </c>
-      <c r="G52" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H52" s="108" t="s">
-        <v>185</v>
-      </c>
-      <c r="I52" s="62" t="s">
-        <v>265</v>
-      </c>
-      <c r="J52" s="59" t="s">
-        <v>216</v>
-      </c>
-      <c r="K52" s="56">
-        <v>1</v>
-      </c>
-      <c r="L52" s="30">
+      <c r="C52" s="52" t="s">
+        <v>46</v>
+      </c>
+      <c r="D52" s="61" t="s">
+        <v>86</v>
+      </c>
+      <c r="E52" s="52" t="s">
+        <v>199</v>
+      </c>
+      <c r="F52" s="61" t="s">
+        <v>118</v>
+      </c>
+      <c r="G52" s="58" t="s">
+        <v>200</v>
+      </c>
+      <c r="H52" s="99" t="s">
+        <v>172</v>
+      </c>
+      <c r="I52" s="61" t="s">
+        <v>249</v>
+      </c>
+      <c r="J52" s="52" t="s">
+        <v>196</v>
+      </c>
+      <c r="K52" s="55">
+        <v>2</v>
+      </c>
+      <c r="L52" s="31">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="M52" s="30">
         <v>10</v>
       </c>
-      <c r="N52" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O52" s="34">
-        <v>2.0400000000000001E-2</v>
-      </c>
-      <c r="P52" s="34">
+      <c r="M52" s="31">
+        <v>11</v>
+      </c>
+      <c r="N52" s="70" t="s">
+        <v>209</v>
+      </c>
+      <c r="O52" s="35">
+        <v>0.27650000000000002</v>
+      </c>
+      <c r="P52" s="35">
         <f t="shared" si="2"/>
-        <v>0.20400000000000001</v>
-      </c>
-      <c r="Q52" s="34"/>
-      <c r="R52" s="34"/>
+        <v>3.0415000000000001</v>
+      </c>
+      <c r="Q52" s="35"/>
+      <c r="R52" s="35"/>
     </row>
     <row r="53" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A53" s="1"/>
@@ -4688,266 +4689,212 @@
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="C53" s="52" t="s">
-        <v>54</v>
-      </c>
-      <c r="D53" s="61" t="s">
-        <v>96</v>
-      </c>
-      <c r="E53" s="52" t="s">
-        <v>214</v>
-      </c>
-      <c r="F53" s="61" t="s">
-        <v>129</v>
-      </c>
-      <c r="G53" s="58" t="s">
-        <v>215</v>
-      </c>
-      <c r="H53" s="107" t="s">
-        <v>186</v>
-      </c>
-      <c r="I53" s="61" t="s">
-        <v>266</v>
-      </c>
-      <c r="J53" s="52" t="s">
-        <v>211</v>
-      </c>
-      <c r="K53" s="55">
-        <v>2</v>
-      </c>
-      <c r="L53" s="31">
+      <c r="C53" s="53" t="s">
+        <v>47</v>
+      </c>
+      <c r="D53" s="62" t="s">
+        <v>87</v>
+      </c>
+      <c r="E53" s="53" t="s">
+        <v>199</v>
+      </c>
+      <c r="F53" s="62" t="s">
+        <v>119</v>
+      </c>
+      <c r="G53" s="59" t="s">
+        <v>200</v>
+      </c>
+      <c r="H53" s="100" t="s">
+        <v>172</v>
+      </c>
+      <c r="I53" s="62" t="s">
+        <v>250</v>
+      </c>
+      <c r="J53" s="53" t="s">
+        <v>197</v>
+      </c>
+      <c r="K53" s="56">
+        <v>1</v>
+      </c>
+      <c r="L53" s="30">
         <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="M53" s="30">
         <v>10</v>
       </c>
-      <c r="M53" s="31">
-        <v>11</v>
-      </c>
-      <c r="N53" s="70" t="s">
-        <v>224</v>
-      </c>
-      <c r="O53" s="35">
-        <v>0.27650000000000002</v>
-      </c>
-      <c r="P53" s="35">
+      <c r="N53" s="71" t="s">
+        <v>209</v>
+      </c>
+      <c r="O53" s="34">
+        <v>9.7100000000000006E-2</v>
+      </c>
+      <c r="P53" s="34">
         <f t="shared" si="2"/>
-        <v>3.0415000000000001</v>
-      </c>
-      <c r="Q53" s="35"/>
-      <c r="R53" s="35"/>
-    </row>
-    <row r="54" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
+        <v>0.97100000000000009</v>
+      </c>
+      <c r="Q53" s="34"/>
+      <c r="R53" s="34"/>
+    </row>
+    <row r="54" spans="1:18" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="1"/>
       <c r="B54" s="78">
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
-      <c r="C54" s="53" t="s">
-        <v>55</v>
-      </c>
-      <c r="D54" s="62" t="s">
-        <v>97</v>
-      </c>
-      <c r="E54" s="53" t="s">
-        <v>214</v>
-      </c>
-      <c r="F54" s="62" t="s">
-        <v>130</v>
-      </c>
-      <c r="G54" s="59" t="s">
-        <v>215</v>
-      </c>
-      <c r="H54" s="108" t="s">
-        <v>186</v>
-      </c>
-      <c r="I54" s="62" t="s">
-        <v>267</v>
-      </c>
-      <c r="J54" s="53" t="s">
-        <v>212</v>
-      </c>
-      <c r="K54" s="56">
+      <c r="C54" s="68" t="s">
+        <v>48</v>
+      </c>
+      <c r="D54" s="64" t="s">
+        <v>88</v>
+      </c>
+      <c r="E54" s="110" t="s">
+        <v>199</v>
+      </c>
+      <c r="F54" s="64" t="s">
+        <v>120</v>
+      </c>
+      <c r="G54" s="107" t="s">
+        <v>200</v>
+      </c>
+      <c r="H54" s="105" t="s">
+        <v>173</v>
+      </c>
+      <c r="I54" s="64" t="s">
+        <v>251</v>
+      </c>
+      <c r="J54" s="110" t="s">
+        <v>198</v>
+      </c>
+      <c r="K54" s="57">
         <v>1</v>
       </c>
-      <c r="L54" s="30">
+      <c r="L54" s="45">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M54" s="30">
+      <c r="M54" s="45">
         <v>10</v>
       </c>
-      <c r="N54" s="71" t="s">
-        <v>224</v>
-      </c>
-      <c r="O54" s="34">
-        <v>9.7100000000000006E-2</v>
-      </c>
-      <c r="P54" s="34">
-        <f t="shared" si="2"/>
-        <v>0.97100000000000009</v>
-      </c>
-      <c r="Q54" s="34"/>
-      <c r="R54" s="34"/>
-    </row>
-    <row r="55" spans="1:18" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="1"/>
-      <c r="B55" s="78">
-        <f t="shared" si="0"/>
-        <v>46</v>
-      </c>
-      <c r="C55" s="68" t="s">
-        <v>56</v>
-      </c>
-      <c r="D55" s="64" t="s">
-        <v>98</v>
-      </c>
-      <c r="E55" s="118" t="s">
-        <v>214</v>
-      </c>
-      <c r="F55" s="64" t="s">
-        <v>131</v>
-      </c>
-      <c r="G55" s="115" t="s">
-        <v>215</v>
-      </c>
-      <c r="H55" s="113" t="s">
-        <v>187</v>
-      </c>
-      <c r="I55" s="64" t="s">
-        <v>268</v>
-      </c>
-      <c r="J55" s="68" t="s">
-        <v>213</v>
-      </c>
-      <c r="K55" s="57">
-        <v>1</v>
-      </c>
-      <c r="L55" s="45">
-        <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-      <c r="M55" s="45">
-        <v>10</v>
-      </c>
-      <c r="N55" s="73" t="s">
-        <v>224</v>
-      </c>
-      <c r="O55" s="46">
+      <c r="N54" s="73" t="s">
+        <v>209</v>
+      </c>
+      <c r="O54" s="46">
         <v>0.13439999999999999</v>
       </c>
-      <c r="P55" s="46">
+      <c r="P54" s="46">
         <f t="shared" si="2"/>
         <v>1.3439999999999999</v>
       </c>
-      <c r="Q55" s="46"/>
-      <c r="R55" s="46"/>
+      <c r="Q54" s="46"/>
+      <c r="R54" s="46"/>
+    </row>
+    <row r="55" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="1"/>
+      <c r="B55" s="47"/>
+      <c r="C55" s="48" t="s">
+        <v>5</v>
+      </c>
+      <c r="D55" s="49"/>
+      <c r="E55" s="50"/>
+      <c r="F55" s="66"/>
+      <c r="G55" s="66"/>
+      <c r="H55" s="66"/>
+      <c r="I55" s="66"/>
+      <c r="J55" s="66"/>
+      <c r="K55" s="66"/>
+      <c r="L55" s="66"/>
+      <c r="M55" s="115" t="s">
+        <v>260</v>
+      </c>
+      <c r="N55" s="116"/>
+      <c r="O55" s="116"/>
+      <c r="P55" s="75">
+        <f>SUM(P10:P54)</f>
+        <v>155.34110000000001</v>
+      </c>
+      <c r="Q55" s="66"/>
+      <c r="R55" s="67"/>
     </row>
     <row r="56" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="1"/>
-      <c r="B56" s="47"/>
-      <c r="C56" s="48" t="s">
-        <v>5</v>
-      </c>
-      <c r="D56" s="49"/>
-      <c r="E56" s="50"/>
-      <c r="F56" s="66"/>
-      <c r="G56" s="66"/>
-      <c r="H56" s="66"/>
-      <c r="I56" s="66"/>
-      <c r="J56" s="66"/>
-      <c r="K56" s="66"/>
-      <c r="L56" s="66"/>
-      <c r="M56" s="101" t="s">
-        <v>277</v>
-      </c>
-      <c r="N56" s="102"/>
-      <c r="O56" s="102"/>
-      <c r="P56" s="75">
-        <f>SUM(P10:P55)</f>
-        <v>156.01360000000003</v>
-      </c>
-      <c r="Q56" s="66"/>
-      <c r="R56" s="67"/>
-    </row>
-    <row r="57" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="1"/>
-      <c r="B57" s="24"/>
-      <c r="C57" s="8" t="s">
+      <c r="B56" s="24"/>
+      <c r="C56" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="D57" s="9"/>
-      <c r="E57" s="9"/>
-      <c r="F57" s="43"/>
-      <c r="G57" s="43"/>
-      <c r="H57" s="43"/>
-      <c r="I57" s="43"/>
-      <c r="J57" s="43"/>
-      <c r="K57" s="43"/>
-      <c r="L57" s="43"/>
-      <c r="M57" s="101" t="s">
-        <v>278</v>
-      </c>
-      <c r="N57" s="102"/>
-      <c r="O57" s="102"/>
-      <c r="P57" s="74">
-        <f>P56/5</f>
-        <v>31.202720000000006</v>
-      </c>
-      <c r="Q57" s="43"/>
-      <c r="R57" s="44"/>
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="43"/>
+      <c r="G56" s="43"/>
+      <c r="H56" s="43"/>
+      <c r="I56" s="43"/>
+      <c r="J56" s="43"/>
+      <c r="K56" s="43"/>
+      <c r="L56" s="43"/>
+      <c r="M56" s="115" t="s">
+        <v>261</v>
+      </c>
+      <c r="N56" s="116"/>
+      <c r="O56" s="116"/>
+      <c r="P56" s="74">
+        <f>P55/5</f>
+        <v>31.068220000000004</v>
+      </c>
+      <c r="Q56" s="43"/>
+      <c r="R56" s="44"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="R3:R8"/>
     <mergeCell ref="J2:R2"/>
+    <mergeCell ref="M55:O55"/>
     <mergeCell ref="M56:O56"/>
-    <mergeCell ref="M57:O57"/>
     <mergeCell ref="J1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="N10" r:id="rId1" xr:uid="{89FE49F2-489B-4F8E-8442-F4F08D2A71B9}"/>
-    <hyperlink ref="N11" r:id="rId2" xr:uid="{B2C94EB8-361E-4059-912A-7E08189FF588}"/>
-    <hyperlink ref="N12" r:id="rId3" xr:uid="{C19BE0B1-F1F1-4F20-B4BD-E9C636ECF5F4}"/>
-    <hyperlink ref="N14" r:id="rId4" xr:uid="{7F307109-CE66-4E56-B927-F44D4A7D1544}"/>
-    <hyperlink ref="N13" r:id="rId5" xr:uid="{452140BD-B707-4DD6-97FD-06A0408D0F5E}"/>
-    <hyperlink ref="N15" r:id="rId6" xr:uid="{567837A6-FAC1-4EE4-8093-25DE77AB4C76}"/>
-    <hyperlink ref="N16" r:id="rId7" xr:uid="{84DDAAD3-0D88-427C-B37F-EF4F7D64C3F9}"/>
-    <hyperlink ref="N17" r:id="rId8" xr:uid="{0F02C980-61A3-4E84-B81B-D6711E4DA791}"/>
-    <hyperlink ref="N18" r:id="rId9" xr:uid="{1F51A281-7903-4DE5-9D43-C8D611F3E5B3}"/>
-    <hyperlink ref="N19" r:id="rId10" xr:uid="{F9BCC43B-5974-4F21-BB56-696E568D40F2}"/>
-    <hyperlink ref="N20" r:id="rId11" xr:uid="{71BDBDEC-A643-4EE2-AB8B-77BCE9EFCD5F}"/>
-    <hyperlink ref="N21" r:id="rId12" xr:uid="{66E014D8-15DF-496D-B3EF-4C478897BEE9}"/>
-    <hyperlink ref="N22" r:id="rId13" xr:uid="{977C37EA-9C73-4C4C-B8BA-458124D4F10B}"/>
-    <hyperlink ref="N24" r:id="rId14" xr:uid="{FEE6FFE2-6B3E-4EE5-9854-876785A32929}"/>
-    <hyperlink ref="N27" r:id="rId15" xr:uid="{7524F555-50E1-47E0-AF8E-5BC45B838FFE}"/>
-    <hyperlink ref="N28" r:id="rId16" xr:uid="{E0EBA58F-E359-4BCB-A2C9-9C49D150A629}"/>
-    <hyperlink ref="N29" r:id="rId17" xr:uid="{30630BC0-7DB5-4073-8F22-E28F5B42FCE1}"/>
-    <hyperlink ref="N32" r:id="rId18" xr:uid="{D7F6D37C-1F7B-418B-9244-5EC422B2C736}"/>
-    <hyperlink ref="N30" r:id="rId19" xr:uid="{7EC7E3F1-93CD-45A5-BAEC-2E96006DD4BC}"/>
-    <hyperlink ref="N31" r:id="rId20" xr:uid="{DAFC4B5E-88AC-4044-8DE5-E6B95F9FA94C}"/>
-    <hyperlink ref="N33" r:id="rId21" xr:uid="{FC25DD16-B062-4971-87F3-FBBA153342C7}"/>
-    <hyperlink ref="N34" r:id="rId22" xr:uid="{BA75FE37-D1AE-4A06-A7D6-2FC24E19A57B}"/>
-    <hyperlink ref="N37" r:id="rId23" xr:uid="{F2FCE814-68EB-42CA-B801-47EACCC9D840}"/>
-    <hyperlink ref="N38" r:id="rId24" xr:uid="{B8B83BF6-E82D-4A6D-9C89-2F85CAB04646}"/>
-    <hyperlink ref="N42" r:id="rId25" xr:uid="{377F7D05-CD56-46CE-86C7-8359A58D6174}"/>
-    <hyperlink ref="N39" r:id="rId26" xr:uid="{5BC7FB0B-A7A9-4A4F-B0AF-D93D90BD0257}"/>
-    <hyperlink ref="N40" r:id="rId27" xr:uid="{42342919-596A-4C59-8816-01D385B759CB}"/>
-    <hyperlink ref="N41" r:id="rId28" xr:uid="{5D8F6C78-4114-4B09-9296-33D8E0033965}"/>
-    <hyperlink ref="N44" r:id="rId29" xr:uid="{30A94DA1-5BD4-4155-A48B-F08C168CF099}"/>
-    <hyperlink ref="N46" r:id="rId30" xr:uid="{C3F3FC15-3DA9-4B1A-84AC-5A582D205C55}"/>
-    <hyperlink ref="N48" r:id="rId31" xr:uid="{3A097DB9-C3B3-436E-8B87-273AE27C3FB3}"/>
-    <hyperlink ref="N50" r:id="rId32" xr:uid="{0763754B-803A-440F-9046-E7656CF9DB82}"/>
-    <hyperlink ref="N51" r:id="rId33" xr:uid="{4C3FCDA1-65D2-4395-9426-3E1F29BD784A}"/>
-    <hyperlink ref="N52" r:id="rId34" xr:uid="{A4B71E3E-7A98-4CCB-A3C2-8B949A858D06}"/>
-    <hyperlink ref="N53" r:id="rId35" xr:uid="{8DCBF280-B1E4-481C-8762-45E69BB689C9}"/>
-    <hyperlink ref="N54" r:id="rId36" xr:uid="{9D7C6330-6521-4E77-B082-7293A2D402F7}"/>
-    <hyperlink ref="N55" r:id="rId37" xr:uid="{60E4F958-BD03-4950-AA1A-E5483E7B8267}"/>
-    <hyperlink ref="N36" r:id="rId38" xr:uid="{019A488B-4FF7-4C4E-B4AC-B360044B8376}"/>
-    <hyperlink ref="N23" r:id="rId39" xr:uid="{83A2C1C1-8C25-4D67-A480-302431668718}"/>
-    <hyperlink ref="N25" r:id="rId40" xr:uid="{30D22A24-3F30-4E99-967B-FA4F0FA9B8E8}"/>
-    <hyperlink ref="N35" r:id="rId41" xr:uid="{E6D3A492-9D47-4832-8671-ED5B61C9ACB1}"/>
+    <hyperlink ref="N10" r:id="rId1"/>
+    <hyperlink ref="N11" r:id="rId2"/>
+    <hyperlink ref="N12" r:id="rId3"/>
+    <hyperlink ref="N14" r:id="rId4"/>
+    <hyperlink ref="N13" r:id="rId5"/>
+    <hyperlink ref="N15" r:id="rId6"/>
+    <hyperlink ref="N16" r:id="rId7"/>
+    <hyperlink ref="N18" r:id="rId8"/>
+    <hyperlink ref="N19" r:id="rId9"/>
+    <hyperlink ref="N20" r:id="rId10"/>
+    <hyperlink ref="N21" r:id="rId11"/>
+    <hyperlink ref="N22" r:id="rId12"/>
+    <hyperlink ref="N23" r:id="rId13"/>
+    <hyperlink ref="N25" r:id="rId14"/>
+    <hyperlink ref="N28" r:id="rId15"/>
+    <hyperlink ref="N29" r:id="rId16"/>
+    <hyperlink ref="N32" r:id="rId17"/>
+    <hyperlink ref="N30" r:id="rId18"/>
+    <hyperlink ref="N31" r:id="rId19"/>
+    <hyperlink ref="N33" r:id="rId20"/>
+    <hyperlink ref="N34" r:id="rId21"/>
+    <hyperlink ref="N37" r:id="rId22"/>
+    <hyperlink ref="N41" r:id="rId23"/>
+    <hyperlink ref="N38" r:id="rId24"/>
+    <hyperlink ref="N39" r:id="rId25"/>
+    <hyperlink ref="N40" r:id="rId26"/>
+    <hyperlink ref="N43" r:id="rId27"/>
+    <hyperlink ref="N45" r:id="rId28"/>
+    <hyperlink ref="N47" r:id="rId29"/>
+    <hyperlink ref="N49" r:id="rId30"/>
+    <hyperlink ref="N50" r:id="rId31"/>
+    <hyperlink ref="N51" r:id="rId32"/>
+    <hyperlink ref="N52" r:id="rId33"/>
+    <hyperlink ref="N53" r:id="rId34"/>
+    <hyperlink ref="N54" r:id="rId35"/>
+    <hyperlink ref="N36" r:id="rId36"/>
+    <hyperlink ref="N24" r:id="rId37"/>
+    <hyperlink ref="N26" r:id="rId38"/>
+    <hyperlink ref="N35" r:id="rId39"/>
+    <hyperlink ref="N17" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId42"/>
-  <drawing r:id="rId43"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId41"/>
+  <drawing r:id="rId42"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
custom supplier quotes added #70
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Control-Board/eSpark_BOM-Control-Board.xlsx
+++ b/Deliverables/BOM/Control-Board/eSpark_BOM-Control-Board.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25225"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BDC7446-3BFB-49C3-9C45-EF973E40F11B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="293">
   <si>
     <t>Component list</t>
   </si>
@@ -800,12 +799,6 @@
     <t>--------</t>
   </si>
   <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reviewer Remarks </t>
-  </si>
-  <si>
     <t>-------</t>
   </si>
   <si>
@@ -903,18 +896,30 @@
   </si>
   <si>
     <t>DO NOT MOUNT</t>
+  </si>
+  <si>
+    <t>Remarks (Iftikhar)</t>
+  </si>
+  <si>
+    <t>Remarks (Faizan)</t>
+  </si>
+  <si>
+    <t>Quote added from Lulu</t>
+  </si>
+  <si>
+    <t>Quote changed after receiving better rates from Lulu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1087,6 +1092,23 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <strike/>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -1514,7 +1536,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="137">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1878,6 +1900,27 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="23" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="7" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="6" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1918,7 +1961,7 @@
         <xdr:cNvPr id="9" name="Picture 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7484868C-6378-4A14-8499-0201EF52182D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{7484868C-6378-4A14-8499-0201EF52182D}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2214,7 +2257,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:R56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2235,7 +2278,7 @@
     <col min="15" max="15" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="42.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="36" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2440,7 +2483,7 @@
         <v>205</v>
       </c>
       <c r="L9" s="32" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="M9" s="32" t="s">
         <v>206</v>
@@ -2452,13 +2495,13 @@
         <v>208</v>
       </c>
       <c r="P9" s="32" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="Q9" s="32" t="s">
-        <v>256</v>
+        <v>289</v>
       </c>
       <c r="R9" s="32" t="s">
-        <v>257</v>
+        <v>290</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
@@ -2521,7 +2564,7 @@
         <v>2</v>
       </c>
       <c r="C11" s="52" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="D11" s="61" t="s">
         <v>51</v>
@@ -2680,7 +2723,7 @@
         <v>5</v>
       </c>
       <c r="C14" s="53" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D14" s="62" t="s">
         <v>54</v>
@@ -2733,7 +2776,7 @@
         <v>6</v>
       </c>
       <c r="C15" s="52" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D15" s="61" t="s">
         <v>55</v>
@@ -2839,28 +2882,28 @@
         <v>8</v>
       </c>
       <c r="C17" s="53" t="s">
+        <v>279</v>
+      </c>
+      <c r="D17" s="62" t="s">
+        <v>280</v>
+      </c>
+      <c r="E17" s="53" t="s">
         <v>281</v>
       </c>
-      <c r="D17" s="62" t="s">
+      <c r="F17" s="62" t="s">
         <v>282</v>
-      </c>
-      <c r="E17" s="53" t="s">
-        <v>283</v>
-      </c>
-      <c r="F17" s="62" t="s">
-        <v>284</v>
       </c>
       <c r="G17" s="59" t="s">
         <v>200</v>
       </c>
       <c r="H17" s="62" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="I17" s="110" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J17" s="53" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="K17" s="56">
         <v>1</v>
@@ -2891,7 +2934,7 @@
         <v>9</v>
       </c>
       <c r="C18" s="52" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D18" s="61" t="s">
         <v>218</v>
@@ -3102,52 +3145,52 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="52" t="s">
+      <c r="C22" s="114" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="61" t="s">
+      <c r="D22" s="107" t="s">
         <v>60</v>
       </c>
-      <c r="E22" s="52" t="s">
+      <c r="E22" s="114" t="s">
         <v>199</v>
       </c>
-      <c r="F22" s="61" t="s">
+      <c r="F22" s="107" t="s">
         <v>95</v>
       </c>
-      <c r="G22" s="58" t="s">
+      <c r="G22" s="116" t="s">
         <v>200</v>
       </c>
-      <c r="H22" s="99" t="s">
+      <c r="H22" s="130" t="s">
         <v>155</v>
       </c>
-      <c r="I22" s="61" t="s">
+      <c r="I22" s="107" t="s">
         <v>223</v>
       </c>
-      <c r="J22" s="58" t="s">
+      <c r="J22" s="116" t="s">
         <v>200</v>
       </c>
-      <c r="K22" s="55">
+      <c r="K22" s="118">
         <v>1</v>
       </c>
-      <c r="L22" s="31">
+      <c r="L22" s="119">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="M22" s="31">
+      <c r="M22" s="119">
         <v>20</v>
       </c>
-      <c r="N22" s="70" t="s">
+      <c r="N22" s="131" t="s">
         <v>209</v>
       </c>
-      <c r="O22" s="35">
-        <v>4.8399999999999999E-2</v>
-      </c>
-      <c r="P22" s="35">
+      <c r="O22" s="132"/>
+      <c r="P22" s="132">
         <f t="shared" si="2"/>
-        <v>0.96799999999999997</v>
+        <v>0</v>
       </c>
       <c r="Q22" s="35"/>
-      <c r="R22" s="35"/>
+      <c r="R22" s="134" t="s">
+        <v>288</v>
+      </c>
     </row>
     <row r="23" spans="1:18" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
@@ -3212,22 +3255,22 @@
         <v>20</v>
       </c>
       <c r="D24" s="97" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E24" s="52" t="s">
         <v>97</v>
       </c>
       <c r="F24" s="63" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="G24" s="58" t="s">
         <v>200</v>
       </c>
       <c r="H24" s="99" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="I24" s="61" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="J24" s="58" t="s">
         <v>200</v>
@@ -3274,7 +3317,7 @@
         <v>98</v>
       </c>
       <c r="G25" s="59" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="H25" s="100" t="s">
         <v>153</v>
@@ -3318,22 +3361,22 @@
         <v>22</v>
       </c>
       <c r="D26" s="63" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="E26" s="52" t="s">
         <v>99</v>
       </c>
       <c r="F26" s="63" t="s">
+        <v>265</v>
+      </c>
+      <c r="G26" s="58" t="s">
+        <v>256</v>
+      </c>
+      <c r="H26" s="99" t="s">
+        <v>263</v>
+      </c>
+      <c r="I26" s="61" t="s">
         <v>267</v>
-      </c>
-      <c r="G26" s="58" t="s">
-        <v>258</v>
-      </c>
-      <c r="H26" s="99" t="s">
-        <v>265</v>
-      </c>
-      <c r="I26" s="61" t="s">
-        <v>269</v>
       </c>
       <c r="J26" s="58" t="s">
         <v>200</v>
@@ -3380,13 +3423,13 @@
         <v>100</v>
       </c>
       <c r="G27" s="96" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H27" s="101" t="s">
         <v>152</v>
       </c>
       <c r="I27" s="90" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="J27" s="88" t="s">
         <v>184</v>
@@ -3399,18 +3442,24 @@
         <v>5</v>
       </c>
       <c r="M27" s="92">
-        <v>7</v>
-      </c>
-      <c r="N27" s="93"/>
-      <c r="O27" s="94"/>
-      <c r="P27" s="94">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="N27" s="93" t="s">
+        <v>201</v>
+      </c>
+      <c r="O27" s="94">
+        <v>0.48</v>
+      </c>
+      <c r="P27" s="135">
+        <f>O27*M27</f>
+        <v>2.88</v>
       </c>
       <c r="Q27" s="95" t="s">
-        <v>277</v>
-      </c>
-      <c r="R27" s="94"/>
+        <v>275</v>
+      </c>
+      <c r="R27" s="133" t="s">
+        <v>291</v>
+      </c>
     </row>
     <row r="28" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A28" s="1"/>
@@ -3791,22 +3840,22 @@
         <v>31</v>
       </c>
       <c r="D35" s="61" t="s">
+        <v>268</v>
+      </c>
+      <c r="E35" s="52" t="s">
+        <v>269</v>
+      </c>
+      <c r="F35" s="61" t="s">
         <v>270</v>
-      </c>
-      <c r="E35" s="52" t="s">
-        <v>271</v>
-      </c>
-      <c r="F35" s="61" t="s">
-        <v>272</v>
       </c>
       <c r="G35" s="58" t="s">
         <v>200</v>
       </c>
       <c r="H35" s="102" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="I35" s="61" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="J35" s="52" t="s">
         <v>189</v>
@@ -3947,7 +3996,7 @@
         <v>29</v>
       </c>
       <c r="C38" s="52" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D38" s="61" t="s">
         <v>72</v>
@@ -4200,7 +4249,7 @@
         <v>201</v>
       </c>
       <c r="Q42" s="121" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="R42" s="65"/>
     </row>
@@ -4211,7 +4260,7 @@
         <v>34</v>
       </c>
       <c r="C43" s="53" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D43" s="62" t="s">
         <v>77</v>
@@ -4297,16 +4346,22 @@
       <c r="M44" s="92">
         <v>6</v>
       </c>
-      <c r="N44" s="93"/>
-      <c r="O44" s="94"/>
-      <c r="P44" s="94">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="N44" s="93" t="s">
+        <v>201</v>
+      </c>
+      <c r="O44" s="94">
+        <v>3.94</v>
+      </c>
+      <c r="P44" s="135">
+        <f>O44*M44</f>
+        <v>23.64</v>
       </c>
       <c r="Q44" s="95" t="s">
-        <v>277</v>
-      </c>
-      <c r="R44" s="94"/>
+        <v>275</v>
+      </c>
+      <c r="R44" s="133" t="s">
+        <v>291</v>
+      </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" s="1"/>
@@ -4401,14 +4456,20 @@
       <c r="M46" s="92">
         <v>6</v>
       </c>
-      <c r="N46" s="93"/>
-      <c r="O46" s="94"/>
+      <c r="N46" s="93" t="s">
+        <v>201</v>
+      </c>
+      <c r="O46" s="94">
+        <v>1.575</v>
+      </c>
       <c r="P46" s="94">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>9.4499999999999993</v>
       </c>
       <c r="Q46" s="95"/>
-      <c r="R46" s="94"/>
+      <c r="R46" s="133" t="s">
+        <v>291</v>
+      </c>
     </row>
     <row r="47" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A47" s="1"/>
@@ -4451,19 +4512,21 @@
         <v>6</v>
       </c>
       <c r="N47" s="85" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="O47" s="86">
-        <v>12.0063</v>
+        <v>7.88</v>
       </c>
       <c r="P47" s="86">
         <f t="shared" si="2"/>
-        <v>72.037800000000004</v>
+        <v>47.28</v>
       </c>
       <c r="Q47" s="87" t="s">
-        <v>275</v>
-      </c>
-      <c r="R47" s="86"/>
+        <v>273</v>
+      </c>
+      <c r="R47" s="136" t="s">
+        <v>292</v>
+      </c>
     </row>
     <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" s="1"/>
@@ -4505,16 +4568,22 @@
       <c r="M48" s="92">
         <v>6</v>
       </c>
-      <c r="N48" s="93"/>
-      <c r="O48" s="94"/>
+      <c r="N48" s="93" t="s">
+        <v>201</v>
+      </c>
+      <c r="O48" s="94">
+        <v>12.6</v>
+      </c>
       <c r="P48" s="94">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>75.599999999999994</v>
       </c>
       <c r="Q48" s="95" t="s">
-        <v>277</v>
-      </c>
-      <c r="R48" s="94"/>
+        <v>275</v>
+      </c>
+      <c r="R48" s="133" t="s">
+        <v>291</v>
+      </c>
     </row>
     <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" s="1"/>
@@ -4850,13 +4919,13 @@
       <c r="K55" s="66"/>
       <c r="L55" s="66"/>
       <c r="M55" s="126" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="N55" s="127"/>
       <c r="O55" s="127"/>
       <c r="P55" s="75">
         <f>SUM(P10:P54)</f>
-        <v>155.6626</v>
+        <v>241.5068</v>
       </c>
       <c r="Q55" s="66"/>
       <c r="R55" s="67"/>
@@ -4877,13 +4946,13 @@
       <c r="K56" s="43"/>
       <c r="L56" s="43"/>
       <c r="M56" s="126" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="N56" s="127"/>
       <c r="O56" s="127"/>
       <c r="P56" s="74">
         <f>P55/5</f>
-        <v>31.13252</v>
+        <v>48.301360000000003</v>
       </c>
       <c r="Q56" s="43"/>
       <c r="R56" s="44"/>
@@ -4897,46 +4966,46 @@
     <mergeCell ref="J1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="N10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="N11" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="N12" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="N14" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="N13" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="N15" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="N16" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="N18" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="N19" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="N20" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="N21" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="N22" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="N23" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="N25" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="N28" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="N29" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="N32" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="N30" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="N31" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="N33" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="N34" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="N37" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="N41" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="N38" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="N39" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="N40" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="N43" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="N45" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="N47" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="N49" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="N50" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="N51" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="N52" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="N53" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="N54" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="N36" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="N24" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="N26" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="N35" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="N17" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="N10" r:id="rId1"/>
+    <hyperlink ref="N11" r:id="rId2"/>
+    <hyperlink ref="N12" r:id="rId3"/>
+    <hyperlink ref="N14" r:id="rId4"/>
+    <hyperlink ref="N13" r:id="rId5"/>
+    <hyperlink ref="N15" r:id="rId6"/>
+    <hyperlink ref="N16" r:id="rId7"/>
+    <hyperlink ref="N18" r:id="rId8"/>
+    <hyperlink ref="N19" r:id="rId9"/>
+    <hyperlink ref="N20" r:id="rId10"/>
+    <hyperlink ref="N21" r:id="rId11"/>
+    <hyperlink ref="N22" r:id="rId12"/>
+    <hyperlink ref="N23" r:id="rId13"/>
+    <hyperlink ref="N25" r:id="rId14"/>
+    <hyperlink ref="N28" r:id="rId15"/>
+    <hyperlink ref="N29" r:id="rId16"/>
+    <hyperlink ref="N32" r:id="rId17"/>
+    <hyperlink ref="N30" r:id="rId18"/>
+    <hyperlink ref="N31" r:id="rId19"/>
+    <hyperlink ref="N33" r:id="rId20"/>
+    <hyperlink ref="N34" r:id="rId21"/>
+    <hyperlink ref="N37" r:id="rId22"/>
+    <hyperlink ref="N41" r:id="rId23"/>
+    <hyperlink ref="N38" r:id="rId24"/>
+    <hyperlink ref="N39" r:id="rId25"/>
+    <hyperlink ref="N40" r:id="rId26"/>
+    <hyperlink ref="N43" r:id="rId27"/>
+    <hyperlink ref="N45" r:id="rId28"/>
+    <hyperlink ref="N47" r:id="rId29" display="LCSC"/>
+    <hyperlink ref="N49" r:id="rId30"/>
+    <hyperlink ref="N50" r:id="rId31"/>
+    <hyperlink ref="N51" r:id="rId32"/>
+    <hyperlink ref="N52" r:id="rId33"/>
+    <hyperlink ref="N53" r:id="rId34"/>
+    <hyperlink ref="N54" r:id="rId35"/>
+    <hyperlink ref="N36" r:id="rId36"/>
+    <hyperlink ref="N24" r:id="rId37"/>
+    <hyperlink ref="N26" r:id="rId38"/>
+    <hyperlink ref="N35" r:id="rId39"/>
+    <hyperlink ref="N17" r:id="rId40"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId41"/>

</xml_diff>

<commit_message>
Discontinued part number changed in LCSC Electrode BOM
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/Control-Board/eSpark_BOM-Control-Board.xlsx
+++ b/Deliverables/BOM/Control-Board/eSpark_BOM-Control-Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\ManarHarake-sEMGDevice\Deliverables\BOM\Control-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67CD9DA3-6257-4937-98B2-352A059D23E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B24F849-96BA-4166-9238-A4B2485374F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2632,7 +2632,7 @@
       <c r="E12" s="53" t="s">
         <v>92</v>
       </c>
-      <c r="F12" s="62" t="s">
+      <c r="F12" s="108" t="s">
         <v>124</v>
       </c>
       <c r="G12" s="59" t="s">

</xml_diff>